<commit_message>
Updated to add team name
</commit_message>
<xml_diff>
--- a/docs/Datathon Project.xlsx
+++ b/docs/Datathon Project.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://uoa-my.sharepoint.com/personal/ghin287_uoa_auckland_ac_nz/Documents/Documents/University/Datathon temp/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{11450F02-EE81-4929-8FBE-319E30382959}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="9" documentId="8_{11450F02-EE81-4929-8FBE-319E30382959}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{59F1E792-5F51-4658-971C-86D2D19E5EB6}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="8" xr2:uid="{B8873715-DDF3-4B00-844B-82E399C3542D}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{B8873715-DDF3-4B00-844B-82E399C3542D}"/>
   </bookViews>
   <sheets>
     <sheet name="Team Overview" sheetId="2" r:id="rId1"/>
@@ -48,7 +48,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1203" uniqueCount="587">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1204" uniqueCount="588">
   <si>
     <t>court</t>
   </si>
@@ -2044,6 +2044,9 @@
   </si>
   <si>
     <t>This is the extraction used by fct_judgment</t>
+  </si>
+  <si>
+    <t>6 Gramss - Team 4</t>
   </si>
 </sst>
 </file>
@@ -2603,7 +2606,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="127">
+  <cellXfs count="128">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -2826,19 +2829,7 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="15" fontId="0" fillId="17" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="19" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="3" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2855,6 +2846,21 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="3" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -2937,16 +2943,16 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -4639,7 +4645,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{70241A6B-2CF1-42DB-9288-7E14FFCD0A5F}">
-  <dimension ref="A1:K36"/>
+  <dimension ref="A1:G36"/>
   <sheetFormatPr defaultColWidth="21.28515625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="25.42578125" customWidth="1"/>
@@ -4649,89 +4655,94 @@
     <col min="6" max="6" width="28.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="54.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="94" t="s">
+    <row r="1" spans="1:7" ht="54.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="90" t="s">
         <v>263</v>
       </c>
-      <c r="B1" s="95"/>
-      <c r="C1" s="95"/>
-      <c r="D1" s="95"/>
-      <c r="E1" s="95"/>
-      <c r="F1" s="95"/>
-    </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="K2" s="7" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="B1" s="91"/>
+      <c r="C1" s="91"/>
+      <c r="D1" s="91"/>
+      <c r="E1" s="91"/>
+      <c r="F1" s="91"/>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="39" t="s">
         <v>78</v>
       </c>
       <c r="B3" s="37" t="s">
         <v>84</v>
       </c>
-      <c r="E3" s="3"/>
+      <c r="D3" s="90" t="s">
+        <v>587</v>
+      </c>
+      <c r="E3" s="127"/>
       <c r="F3" s="3"/>
-      <c r="K3" s="12" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="G3" s="7" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="39" t="s">
         <v>75</v>
       </c>
       <c r="B4" s="40" t="s">
         <v>77</v>
       </c>
-      <c r="E4" s="3"/>
+      <c r="D4" s="90"/>
+      <c r="E4" s="127"/>
       <c r="F4" s="3"/>
-      <c r="K4" s="11" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="G4" s="12" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="39" t="s">
         <v>76</v>
       </c>
       <c r="B5" s="40" t="s">
         <v>312</v>
       </c>
-      <c r="E5" s="3"/>
+      <c r="D5" s="90"/>
+      <c r="E5" s="127"/>
       <c r="F5" s="3"/>
-      <c r="K5" s="10" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="G5" s="11" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="39" t="s">
         <v>68</v>
       </c>
       <c r="B6" s="37" t="s">
         <v>87</v>
       </c>
-      <c r="E6" s="3"/>
+      <c r="D6" s="90"/>
+      <c r="E6" s="127"/>
       <c r="F6" s="3"/>
-    </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="G6" s="10" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="50"/>
       <c r="B7" s="51"/>
-      <c r="E7" s="3"/>
+      <c r="D7" s="90"/>
+      <c r="E7" s="127"/>
       <c r="F7" s="3"/>
     </row>
-    <row r="10" spans="1:11" ht="62.45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="93" t="s">
+    <row r="10" spans="1:7" ht="62.45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="89" t="s">
         <v>290</v>
       </c>
-      <c r="B10" s="93"/>
-      <c r="C10" s="93"/>
-      <c r="D10" s="93" t="s">
+      <c r="B10" s="89"/>
+      <c r="C10" s="89"/>
+      <c r="D10" s="89" t="s">
         <v>291</v>
       </c>
-      <c r="E10" s="93"/>
-      <c r="F10" s="93"/>
-    </row>
-    <row r="11" spans="1:11" ht="27" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E10" s="89"/>
+      <c r="F10" s="89"/>
+    </row>
+    <row r="11" spans="1:7" ht="27" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="56" t="s">
         <v>18</v>
       </c>
@@ -4751,7 +4762,7 @@
         <v>286</v>
       </c>
     </row>
-    <row r="12" spans="1:11" ht="45" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:7" ht="45" x14ac:dyDescent="0.25">
       <c r="A12" s="52" t="s">
         <v>8</v>
       </c>
@@ -4771,7 +4782,7 @@
         <v>264</v>
       </c>
     </row>
-    <row r="13" spans="1:11" ht="75" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:7" ht="75" x14ac:dyDescent="0.25">
       <c r="A13" s="32" t="s">
         <v>9</v>
       </c>
@@ -4791,7 +4802,7 @@
         <v>272</v>
       </c>
     </row>
-    <row r="14" spans="1:11" ht="45" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:7" ht="45" x14ac:dyDescent="0.25">
       <c r="A14" s="32" t="s">
         <v>6</v>
       </c>
@@ -4811,7 +4822,7 @@
         <v>268</v>
       </c>
     </row>
-    <row r="15" spans="1:11" ht="30" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A15" s="32" t="s">
         <v>7</v>
       </c>
@@ -4831,7 +4842,7 @@
         <v>267</v>
       </c>
     </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" s="32" t="s">
         <v>4</v>
       </c>
@@ -4870,10 +4881,10 @@
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A20" s="91" t="s">
+      <c r="A20" s="87" t="s">
         <v>258</v>
       </c>
-      <c r="B20" s="92"/>
+      <c r="B20" s="88"/>
     </row>
     <row r="21" spans="1:6" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="57" t="s">
@@ -4973,11 +4984,12 @@
     </row>
     <row r="36" spans="1:2" ht="14.45" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
-  <mergeCells count="4">
+  <mergeCells count="5">
     <mergeCell ref="A20:B20"/>
     <mergeCell ref="A10:C10"/>
     <mergeCell ref="D10:F10"/>
     <mergeCell ref="A1:F1"/>
+    <mergeCell ref="D3:E7"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="B28" r:id="rId1" display="https://drive.google.com/drive/u/6/folders/1Bw7lSWdOExDDpihTWeozwxtdz5_t1KNN" xr:uid="{CF98AABD-B6DF-493B-8DB4-3101713010F5}"/>
@@ -5245,12 +5257,12 @@
       <c r="C9" s="32" t="s">
         <v>34</v>
       </c>
-      <c r="F9" s="86" t="s">
+      <c r="F9" s="92" t="s">
         <v>308</v>
       </c>
-      <c r="G9" s="87"/>
-      <c r="H9" s="87"/>
-      <c r="I9" s="88"/>
+      <c r="G9" s="93"/>
+      <c r="H9" s="93"/>
+      <c r="I9" s="94"/>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10" s="32">
@@ -5286,60 +5298,60 @@
       </c>
     </row>
     <row r="14" spans="1:9" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B14" s="89" t="s">
+      <c r="B14" s="95" t="s">
         <v>326</v>
       </c>
-      <c r="C14" s="89"/>
+      <c r="C14" s="95"/>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="B15" s="89"/>
-      <c r="C15" s="89"/>
+      <c r="B15" s="95"/>
+      <c r="C15" s="95"/>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="B16" s="89"/>
-      <c r="C16" s="89"/>
+      <c r="B16" s="95"/>
+      <c r="C16" s="95"/>
     </row>
     <row r="17" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B17" s="89"/>
-      <c r="C17" s="89"/>
+      <c r="B17" s="95"/>
+      <c r="C17" s="95"/>
     </row>
     <row r="18" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B18" s="89"/>
-      <c r="C18" s="89"/>
+      <c r="B18" s="95"/>
+      <c r="C18" s="95"/>
     </row>
     <row r="19" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B19" s="89"/>
-      <c r="C19" s="89"/>
+      <c r="B19" s="95"/>
+      <c r="C19" s="95"/>
     </row>
     <row r="20" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B20" s="89"/>
-      <c r="C20" s="89"/>
+      <c r="B20" s="95"/>
+      <c r="C20" s="95"/>
     </row>
     <row r="21" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B21" s="89"/>
-      <c r="C21" s="89"/>
+      <c r="B21" s="95"/>
+      <c r="C21" s="95"/>
     </row>
     <row r="22" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B22" s="89"/>
-      <c r="C22" s="89"/>
+      <c r="B22" s="95"/>
+      <c r="C22" s="95"/>
     </row>
     <row r="23" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B23" s="89"/>
-      <c r="C23" s="89"/>
+      <c r="B23" s="95"/>
+      <c r="C23" s="95"/>
     </row>
     <row r="24" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B24" s="89"/>
-      <c r="C24" s="89"/>
+      <c r="B24" s="95"/>
+      <c r="C24" s="95"/>
     </row>
     <row r="26" spans="2:3" ht="14.45" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="27" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B27" s="3"/>
     </row>
     <row r="28" spans="2:3" ht="72.599999999999994" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B28" s="90" t="s">
+      <c r="B28" s="96" t="s">
         <v>327</v>
       </c>
-      <c r="C28" s="90"/>
+      <c r="C28" s="96"/>
     </row>
     <row r="29" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B29" s="3"/>
@@ -5421,12 +5433,12 @@
       <c r="D2" s="9" t="s">
         <v>87</v>
       </c>
-      <c r="G2" s="97" t="s">
+      <c r="G2" s="98" t="s">
         <v>309</v>
       </c>
-      <c r="H2" s="98"/>
-      <c r="I2" s="98"/>
-      <c r="J2" s="99"/>
+      <c r="H2" s="99"/>
+      <c r="I2" s="99"/>
+      <c r="J2" s="100"/>
     </row>
     <row r="3" spans="2:10" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B3" s="36" t="s">
@@ -5438,10 +5450,10 @@
       <c r="D3" s="9" t="s">
         <v>87</v>
       </c>
-      <c r="G3" s="100"/>
-      <c r="H3" s="101"/>
-      <c r="I3" s="101"/>
-      <c r="J3" s="102"/>
+      <c r="G3" s="101"/>
+      <c r="H3" s="102"/>
+      <c r="I3" s="102"/>
+      <c r="J3" s="103"/>
     </row>
     <row r="4" spans="2:10" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B4" s="36" t="s">
@@ -5453,10 +5465,10 @@
       <c r="D4" s="9" t="s">
         <v>87</v>
       </c>
-      <c r="G4" s="100"/>
-      <c r="H4" s="101"/>
-      <c r="I4" s="101"/>
-      <c r="J4" s="102"/>
+      <c r="G4" s="101"/>
+      <c r="H4" s="102"/>
+      <c r="I4" s="102"/>
+      <c r="J4" s="103"/>
     </row>
     <row r="5" spans="2:10" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B5" s="36" t="s">
@@ -5468,10 +5480,10 @@
       <c r="D5" s="9" t="s">
         <v>87</v>
       </c>
-      <c r="G5" s="103"/>
-      <c r="H5" s="104"/>
-      <c r="I5" s="104"/>
-      <c r="J5" s="105"/>
+      <c r="G5" s="104"/>
+      <c r="H5" s="105"/>
+      <c r="I5" s="105"/>
+      <c r="J5" s="106"/>
     </row>
     <row r="6" spans="2:10" ht="30" x14ac:dyDescent="0.25">
       <c r="B6" s="36" t="s">
@@ -5505,12 +5517,12 @@
       <c r="D8" s="9" t="s">
         <v>87</v>
       </c>
-      <c r="G8" s="106" t="s">
+      <c r="G8" s="107" t="s">
         <v>248</v>
       </c>
-      <c r="H8" s="107"/>
-      <c r="I8" s="107"/>
-      <c r="J8" s="108"/>
+      <c r="H8" s="108"/>
+      <c r="I8" s="108"/>
+      <c r="J8" s="109"/>
     </row>
     <row r="9" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B9" s="36" t="s">
@@ -5522,10 +5534,10 @@
       <c r="D9" s="9" t="s">
         <v>87</v>
       </c>
-      <c r="G9" s="109"/>
-      <c r="H9" s="110"/>
-      <c r="I9" s="110"/>
-      <c r="J9" s="111"/>
+      <c r="G9" s="110"/>
+      <c r="H9" s="111"/>
+      <c r="I9" s="111"/>
+      <c r="J9" s="112"/>
     </row>
     <row r="10" spans="2:10" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B10" s="36" t="s">
@@ -5537,114 +5549,114 @@
       <c r="D10" s="9" t="s">
         <v>87</v>
       </c>
-      <c r="G10" s="109"/>
-      <c r="H10" s="110"/>
-      <c r="I10" s="110"/>
-      <c r="J10" s="111"/>
+      <c r="G10" s="110"/>
+      <c r="H10" s="111"/>
+      <c r="I10" s="111"/>
+      <c r="J10" s="112"/>
     </row>
     <row r="11" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="G11" s="109"/>
-      <c r="H11" s="110"/>
-      <c r="I11" s="110"/>
-      <c r="J11" s="111"/>
+      <c r="G11" s="110"/>
+      <c r="H11" s="111"/>
+      <c r="I11" s="111"/>
+      <c r="J11" s="112"/>
     </row>
     <row r="12" spans="2:10" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="G12" s="112"/>
-      <c r="H12" s="113"/>
-      <c r="I12" s="113"/>
-      <c r="J12" s="114"/>
+      <c r="G12" s="113"/>
+      <c r="H12" s="114"/>
+      <c r="I12" s="114"/>
+      <c r="J12" s="115"/>
     </row>
     <row r="13" spans="2:10" ht="14.45" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="14" spans="2:10" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="G14" s="89" t="s">
+      <c r="G14" s="95" t="s">
         <v>249</v>
       </c>
-      <c r="H14" s="89"/>
-      <c r="I14" s="89"/>
-      <c r="J14" s="89"/>
+      <c r="H14" s="95"/>
+      <c r="I14" s="95"/>
+      <c r="J14" s="95"/>
     </row>
     <row r="15" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="G15" s="89"/>
-      <c r="H15" s="89"/>
-      <c r="I15" s="89"/>
-      <c r="J15" s="89"/>
+      <c r="G15" s="95"/>
+      <c r="H15" s="95"/>
+      <c r="I15" s="95"/>
+      <c r="J15" s="95"/>
     </row>
     <row r="16" spans="2:10" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="G16" s="89"/>
-      <c r="H16" s="89"/>
-      <c r="I16" s="89"/>
-      <c r="J16" s="89"/>
+      <c r="G16" s="95"/>
+      <c r="H16" s="95"/>
+      <c r="I16" s="95"/>
+      <c r="J16" s="95"/>
     </row>
     <row r="17" spans="7:10" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="G17" s="89"/>
-      <c r="H17" s="89"/>
-      <c r="I17" s="89"/>
-      <c r="J17" s="89"/>
+      <c r="G17" s="95"/>
+      <c r="H17" s="95"/>
+      <c r="I17" s="95"/>
+      <c r="J17" s="95"/>
     </row>
     <row r="18" spans="7:10" ht="14.45" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="19" spans="7:10" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="G19" s="89" t="s">
+      <c r="G19" s="95" t="s">
         <v>250</v>
       </c>
-      <c r="H19" s="89"/>
-      <c r="I19" s="89"/>
-      <c r="J19" s="89"/>
+      <c r="H19" s="95"/>
+      <c r="I19" s="95"/>
+      <c r="J19" s="95"/>
     </row>
     <row r="20" spans="7:10" x14ac:dyDescent="0.25">
-      <c r="G20" s="89"/>
-      <c r="H20" s="89"/>
-      <c r="I20" s="89"/>
-      <c r="J20" s="89"/>
+      <c r="G20" s="95"/>
+      <c r="H20" s="95"/>
+      <c r="I20" s="95"/>
+      <c r="J20" s="95"/>
     </row>
     <row r="21" spans="7:10" x14ac:dyDescent="0.25">
-      <c r="G21" s="89"/>
-      <c r="H21" s="89"/>
-      <c r="I21" s="89"/>
-      <c r="J21" s="89"/>
+      <c r="G21" s="95"/>
+      <c r="H21" s="95"/>
+      <c r="I21" s="95"/>
+      <c r="J21" s="95"/>
     </row>
     <row r="22" spans="7:10" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="G22" s="89"/>
-      <c r="H22" s="89"/>
-      <c r="I22" s="89"/>
-      <c r="J22" s="89"/>
+      <c r="G22" s="95"/>
+      <c r="H22" s="95"/>
+      <c r="I22" s="95"/>
+      <c r="J22" s="95"/>
     </row>
     <row r="25" spans="7:10" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="G25" s="96" t="s">
+      <c r="G25" s="97" t="s">
         <v>287</v>
       </c>
-      <c r="H25" s="96"/>
-      <c r="I25" s="96"/>
-      <c r="J25" s="96"/>
+      <c r="H25" s="97"/>
+      <c r="I25" s="97"/>
+      <c r="J25" s="97"/>
     </row>
     <row r="26" spans="7:10" x14ac:dyDescent="0.25">
-      <c r="G26" s="96"/>
-      <c r="H26" s="96"/>
-      <c r="I26" s="96"/>
-      <c r="J26" s="96"/>
+      <c r="G26" s="97"/>
+      <c r="H26" s="97"/>
+      <c r="I26" s="97"/>
+      <c r="J26" s="97"/>
     </row>
     <row r="27" spans="7:10" x14ac:dyDescent="0.25">
-      <c r="G27" s="96"/>
-      <c r="H27" s="96"/>
-      <c r="I27" s="96"/>
-      <c r="J27" s="96"/>
+      <c r="G27" s="97"/>
+      <c r="H27" s="97"/>
+      <c r="I27" s="97"/>
+      <c r="J27" s="97"/>
     </row>
     <row r="28" spans="7:10" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="G28" s="96"/>
-      <c r="H28" s="96"/>
-      <c r="I28" s="96"/>
-      <c r="J28" s="96"/>
+      <c r="G28" s="97"/>
+      <c r="H28" s="97"/>
+      <c r="I28" s="97"/>
+      <c r="J28" s="97"/>
     </row>
     <row r="29" spans="7:10" x14ac:dyDescent="0.25">
-      <c r="G29" s="96"/>
-      <c r="H29" s="96"/>
-      <c r="I29" s="96"/>
-      <c r="J29" s="96"/>
+      <c r="G29" s="97"/>
+      <c r="H29" s="97"/>
+      <c r="I29" s="97"/>
+      <c r="J29" s="97"/>
     </row>
     <row r="30" spans="7:10" x14ac:dyDescent="0.25">
-      <c r="G30" s="96"/>
-      <c r="H30" s="96"/>
-      <c r="I30" s="96"/>
-      <c r="J30" s="96"/>
+      <c r="G30" s="97"/>
+      <c r="H30" s="97"/>
+      <c r="I30" s="97"/>
+      <c r="J30" s="97"/>
     </row>
   </sheetData>
   <mergeCells count="5">
@@ -7274,62 +7286,62 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:37" ht="83.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="118" t="s">
+      <c r="A1" s="119" t="s">
         <v>421</v>
       </c>
-      <c r="B1" s="119"/>
-      <c r="C1" s="119"/>
-      <c r="D1" s="119"/>
-      <c r="E1" s="119"/>
-      <c r="G1" s="119" t="s">
+      <c r="B1" s="120"/>
+      <c r="C1" s="120"/>
+      <c r="D1" s="120"/>
+      <c r="E1" s="120"/>
+      <c r="G1" s="120" t="s">
         <v>328</v>
       </c>
-      <c r="H1" s="119"/>
-      <c r="I1" s="119"/>
-      <c r="J1" s="119"/>
-      <c r="K1" s="119"/>
-      <c r="L1" s="119"/>
-      <c r="M1" s="119"/>
-      <c r="N1" s="119"/>
-      <c r="P1" s="118" t="s">
+      <c r="H1" s="120"/>
+      <c r="I1" s="120"/>
+      <c r="J1" s="120"/>
+      <c r="K1" s="120"/>
+      <c r="L1" s="120"/>
+      <c r="M1" s="120"/>
+      <c r="N1" s="120"/>
+      <c r="P1" s="119" t="s">
         <v>330</v>
       </c>
-      <c r="Q1" s="119"/>
-      <c r="R1" s="119"/>
-      <c r="S1" s="119"/>
-      <c r="T1" s="119"/>
-      <c r="U1" s="119"/>
-      <c r="V1" s="119"/>
-      <c r="W1" s="119"/>
-      <c r="X1" s="119"/>
-      <c r="Y1" s="119"/>
-      <c r="Z1" s="119"/>
-      <c r="AA1" s="119"/>
-      <c r="AB1" s="119"/>
-      <c r="AC1" s="119"/>
-      <c r="AD1" s="119"/>
-      <c r="AE1" s="119"/>
-      <c r="AI1" s="115" t="s">
+      <c r="Q1" s="120"/>
+      <c r="R1" s="120"/>
+      <c r="S1" s="120"/>
+      <c r="T1" s="120"/>
+      <c r="U1" s="120"/>
+      <c r="V1" s="120"/>
+      <c r="W1" s="120"/>
+      <c r="X1" s="120"/>
+      <c r="Y1" s="120"/>
+      <c r="Z1" s="120"/>
+      <c r="AA1" s="120"/>
+      <c r="AB1" s="120"/>
+      <c r="AC1" s="120"/>
+      <c r="AD1" s="120"/>
+      <c r="AE1" s="120"/>
+      <c r="AI1" s="116" t="s">
         <v>310</v>
       </c>
-      <c r="AJ1" s="116"/>
-      <c r="AK1" s="117"/>
+      <c r="AJ1" s="117"/>
+      <c r="AK1" s="118"/>
     </row>
     <row r="33" spans="1:12" ht="42.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="115" t="s">
+      <c r="A33" s="116" t="s">
         <v>329</v>
       </c>
-      <c r="B33" s="116"/>
-      <c r="C33" s="117"/>
-      <c r="F33" s="115" t="s">
+      <c r="B33" s="117"/>
+      <c r="C33" s="118"/>
+      <c r="F33" s="116" t="s">
         <v>417</v>
       </c>
-      <c r="G33" s="116"/>
-      <c r="H33" s="116"/>
-      <c r="I33" s="116"/>
-      <c r="J33" s="116"/>
-      <c r="K33" s="116"/>
-      <c r="L33" s="116"/>
+      <c r="G33" s="117"/>
+      <c r="H33" s="117"/>
+      <c r="I33" s="117"/>
+      <c r="J33" s="117"/>
+      <c r="K33" s="117"/>
+      <c r="L33" s="117"/>
     </row>
   </sheetData>
   <mergeCells count="6">
@@ -8482,96 +8494,96 @@
       </c>
     </row>
     <row r="42" spans="1:24" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A42" s="120" t="s">
+      <c r="A42" s="121" t="s">
         <v>418</v>
       </c>
-      <c r="B42" s="120"/>
-      <c r="C42" s="120"/>
-      <c r="D42" s="120"/>
-      <c r="E42" s="120"/>
-      <c r="F42" s="120"/>
-      <c r="G42" s="120"/>
-      <c r="I42" s="121" t="s">
+      <c r="B42" s="121"/>
+      <c r="C42" s="121"/>
+      <c r="D42" s="121"/>
+      <c r="E42" s="121"/>
+      <c r="F42" s="121"/>
+      <c r="G42" s="121"/>
+      <c r="I42" s="122" t="s">
         <v>419</v>
       </c>
-      <c r="J42" s="122"/>
-      <c r="K42" s="122"/>
-      <c r="L42" s="122"/>
-      <c r="M42" s="122"/>
-      <c r="N42" s="122"/>
-      <c r="O42" s="122"/>
-      <c r="P42" s="122"/>
-      <c r="Q42" s="122"/>
-      <c r="R42" s="122"/>
-      <c r="S42" s="122"/>
-      <c r="T42" s="122"/>
-      <c r="U42" s="122"/>
-      <c r="V42" s="122"/>
-      <c r="W42" s="122"/>
-      <c r="X42" s="122"/>
+      <c r="J42" s="123"/>
+      <c r="K42" s="123"/>
+      <c r="L42" s="123"/>
+      <c r="M42" s="123"/>
+      <c r="N42" s="123"/>
+      <c r="O42" s="123"/>
+      <c r="P42" s="123"/>
+      <c r="Q42" s="123"/>
+      <c r="R42" s="123"/>
+      <c r="S42" s="123"/>
+      <c r="T42" s="123"/>
+      <c r="U42" s="123"/>
+      <c r="V42" s="123"/>
+      <c r="W42" s="123"/>
+      <c r="X42" s="123"/>
     </row>
     <row r="43" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="A43" s="120"/>
-      <c r="B43" s="120"/>
-      <c r="C43" s="120"/>
-      <c r="D43" s="120"/>
-      <c r="E43" s="120"/>
-      <c r="F43" s="120"/>
-      <c r="G43" s="120"/>
-      <c r="I43" s="121"/>
-      <c r="J43" s="122"/>
-      <c r="K43" s="122"/>
-      <c r="L43" s="122"/>
-      <c r="M43" s="122"/>
-      <c r="N43" s="122"/>
-      <c r="O43" s="122"/>
-      <c r="P43" s="122"/>
-      <c r="Q43" s="122"/>
-      <c r="R43" s="122"/>
-      <c r="S43" s="122"/>
-      <c r="T43" s="122"/>
-      <c r="U43" s="122"/>
-      <c r="V43" s="122"/>
-      <c r="W43" s="122"/>
-      <c r="X43" s="122"/>
+      <c r="A43" s="121"/>
+      <c r="B43" s="121"/>
+      <c r="C43" s="121"/>
+      <c r="D43" s="121"/>
+      <c r="E43" s="121"/>
+      <c r="F43" s="121"/>
+      <c r="G43" s="121"/>
+      <c r="I43" s="122"/>
+      <c r="J43" s="123"/>
+      <c r="K43" s="123"/>
+      <c r="L43" s="123"/>
+      <c r="M43" s="123"/>
+      <c r="N43" s="123"/>
+      <c r="O43" s="123"/>
+      <c r="P43" s="123"/>
+      <c r="Q43" s="123"/>
+      <c r="R43" s="123"/>
+      <c r="S43" s="123"/>
+      <c r="T43" s="123"/>
+      <c r="U43" s="123"/>
+      <c r="V43" s="123"/>
+      <c r="W43" s="123"/>
+      <c r="X43" s="123"/>
     </row>
     <row r="60" spans="9:24" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="I60" s="120" t="s">
+      <c r="I60" s="121" t="s">
         <v>420</v>
       </c>
-      <c r="J60" s="120"/>
-      <c r="K60" s="120"/>
-      <c r="L60" s="120"/>
-      <c r="M60" s="120"/>
-      <c r="N60" s="120"/>
-      <c r="O60" s="120"/>
-      <c r="P60" s="120"/>
-      <c r="Q60" s="120"/>
-      <c r="R60" s="120"/>
-      <c r="S60" s="120"/>
-      <c r="T60" s="120"/>
-      <c r="U60" s="120"/>
-      <c r="V60" s="120"/>
-      <c r="W60" s="120"/>
-      <c r="X60" s="120"/>
+      <c r="J60" s="121"/>
+      <c r="K60" s="121"/>
+      <c r="L60" s="121"/>
+      <c r="M60" s="121"/>
+      <c r="N60" s="121"/>
+      <c r="O60" s="121"/>
+      <c r="P60" s="121"/>
+      <c r="Q60" s="121"/>
+      <c r="R60" s="121"/>
+      <c r="S60" s="121"/>
+      <c r="T60" s="121"/>
+      <c r="U60" s="121"/>
+      <c r="V60" s="121"/>
+      <c r="W60" s="121"/>
+      <c r="X60" s="121"/>
     </row>
     <row r="61" spans="9:24" x14ac:dyDescent="0.25">
-      <c r="I61" s="120"/>
-      <c r="J61" s="120"/>
-      <c r="K61" s="120"/>
-      <c r="L61" s="120"/>
-      <c r="M61" s="120"/>
-      <c r="N61" s="120"/>
-      <c r="O61" s="120"/>
-      <c r="P61" s="120"/>
-      <c r="Q61" s="120"/>
-      <c r="R61" s="120"/>
-      <c r="S61" s="120"/>
-      <c r="T61" s="120"/>
-      <c r="U61" s="120"/>
-      <c r="V61" s="120"/>
-      <c r="W61" s="120"/>
-      <c r="X61" s="120"/>
+      <c r="I61" s="121"/>
+      <c r="J61" s="121"/>
+      <c r="K61" s="121"/>
+      <c r="L61" s="121"/>
+      <c r="M61" s="121"/>
+      <c r="N61" s="121"/>
+      <c r="O61" s="121"/>
+      <c r="P61" s="121"/>
+      <c r="Q61" s="121"/>
+      <c r="R61" s="121"/>
+      <c r="S61" s="121"/>
+      <c r="T61" s="121"/>
+      <c r="U61" s="121"/>
+      <c r="V61" s="121"/>
+      <c r="W61" s="121"/>
+      <c r="X61" s="121"/>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -8599,36 +8611,36 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="123" t="s">
+      <c r="A1" s="126" t="s">
         <v>54</v>
       </c>
-      <c r="B1" s="123"/>
-      <c r="C1" s="123"/>
-      <c r="D1" s="123"/>
-      <c r="E1" s="123"/>
+      <c r="B1" s="126"/>
+      <c r="C1" s="126"/>
+      <c r="D1" s="126"/>
+      <c r="E1" s="126"/>
       <c r="H1" s="1"/>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="B3" s="125" t="s">
+      <c r="B3" s="124" t="s">
         <v>429</v>
       </c>
-      <c r="C3" s="126"/>
-      <c r="D3" s="126"/>
-      <c r="E3" s="126"/>
+      <c r="C3" s="125"/>
+      <c r="D3" s="125"/>
+      <c r="E3" s="125"/>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="B4" s="125" t="s">
+      <c r="B4" s="124" t="s">
         <v>430</v>
       </c>
-      <c r="C4" s="126"/>
-      <c r="D4" s="126"/>
-      <c r="E4" s="126"/>
+      <c r="C4" s="125"/>
+      <c r="D4" s="125"/>
+      <c r="E4" s="125"/>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
@@ -8872,23 +8884,23 @@
       <c r="A23" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="B23" s="125" t="s">
+      <c r="B23" s="124" t="s">
         <v>473</v>
       </c>
-      <c r="C23" s="126"/>
-      <c r="D23" s="126"/>
-      <c r="E23" s="126"/>
+      <c r="C23" s="125"/>
+      <c r="D23" s="125"/>
+      <c r="E23" s="125"/>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="B24" s="125" t="s">
+      <c r="B24" s="124" t="s">
         <v>474</v>
       </c>
-      <c r="C24" s="126"/>
-      <c r="D24" s="126"/>
-      <c r="E24" s="126"/>
+      <c r="C24" s="125"/>
+      <c r="D24" s="125"/>
+      <c r="E24" s="125"/>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" s="1" t="s">
@@ -8972,23 +8984,23 @@
       <c r="A32" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="B32" s="125" t="s">
+      <c r="B32" s="124" t="s">
         <v>484</v>
       </c>
-      <c r="C32" s="126"/>
-      <c r="D32" s="126"/>
-      <c r="E32" s="126"/>
+      <c r="C32" s="125"/>
+      <c r="D32" s="125"/>
+      <c r="E32" s="125"/>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A33" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="B33" s="125" t="s">
+      <c r="B33" s="124" t="s">
         <v>485</v>
       </c>
-      <c r="C33" s="126"/>
-      <c r="D33" s="126"/>
-      <c r="E33" s="126"/>
+      <c r="C33" s="125"/>
+      <c r="D33" s="125"/>
+      <c r="E33" s="125"/>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A34" s="1" t="s">
@@ -9042,23 +9054,23 @@
       <c r="A38" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="B38" s="125" t="s">
+      <c r="B38" s="124" t="s">
         <v>487</v>
       </c>
-      <c r="C38" s="126"/>
-      <c r="D38" s="126"/>
-      <c r="E38" s="126"/>
+      <c r="C38" s="125"/>
+      <c r="D38" s="125"/>
+      <c r="E38" s="125"/>
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A39" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="B39" s="125" t="s">
+      <c r="B39" s="124" t="s">
         <v>488</v>
       </c>
-      <c r="C39" s="126"/>
-      <c r="D39" s="126"/>
-      <c r="E39" s="126"/>
+      <c r="C39" s="125"/>
+      <c r="D39" s="125"/>
+      <c r="E39" s="125"/>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A40" s="1" t="s">
@@ -9112,23 +9124,23 @@
       <c r="A44" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="B44" s="125" t="s">
+      <c r="B44" s="124" t="s">
         <v>492</v>
       </c>
-      <c r="C44" s="126"/>
-      <c r="D44" s="126"/>
-      <c r="E44" s="126"/>
+      <c r="C44" s="125"/>
+      <c r="D44" s="125"/>
+      <c r="E44" s="125"/>
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A45" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="B45" s="125" t="s">
+      <c r="B45" s="124" t="s">
         <v>493</v>
       </c>
-      <c r="C45" s="126"/>
-      <c r="D45" s="126"/>
-      <c r="E45" s="126"/>
+      <c r="C45" s="125"/>
+      <c r="D45" s="125"/>
+      <c r="E45" s="125"/>
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A46" s="1" t="s">
@@ -9185,23 +9197,23 @@
       <c r="A50" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="B50" s="125" t="s">
+      <c r="B50" s="124" t="s">
         <v>498</v>
       </c>
-      <c r="C50" s="126"/>
-      <c r="D50" s="126"/>
-      <c r="E50" s="126"/>
+      <c r="C50" s="125"/>
+      <c r="D50" s="125"/>
+      <c r="E50" s="125"/>
     </row>
     <row r="51" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A51" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="B51" s="125" t="s">
+      <c r="B51" s="124" t="s">
         <v>499</v>
       </c>
-      <c r="C51" s="126"/>
-      <c r="D51" s="126"/>
-      <c r="E51" s="126"/>
+      <c r="C51" s="125"/>
+      <c r="D51" s="125"/>
+      <c r="E51" s="125"/>
     </row>
     <row r="52" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A52" s="1" t="s">
@@ -9280,23 +9292,23 @@
       <c r="A58" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="B58" s="125" t="s">
+      <c r="B58" s="124" t="s">
         <v>506</v>
       </c>
-      <c r="C58" s="126"/>
-      <c r="D58" s="126"/>
-      <c r="E58" s="126"/>
+      <c r="C58" s="125"/>
+      <c r="D58" s="125"/>
+      <c r="E58" s="125"/>
     </row>
     <row r="59" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A59" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="B59" s="125" t="s">
+      <c r="B59" s="124" t="s">
         <v>507</v>
       </c>
-      <c r="C59" s="126"/>
-      <c r="D59" s="126"/>
-      <c r="E59" s="126"/>
+      <c r="C59" s="125"/>
+      <c r="D59" s="125"/>
+      <c r="E59" s="125"/>
     </row>
     <row r="60" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A60" s="1" t="s">
@@ -9350,23 +9362,23 @@
       <c r="A64" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="B64" s="125" t="s">
+      <c r="B64" s="124" t="s">
         <v>512</v>
       </c>
-      <c r="C64" s="126"/>
-      <c r="D64" s="126"/>
-      <c r="E64" s="126"/>
+      <c r="C64" s="125"/>
+      <c r="D64" s="125"/>
+      <c r="E64" s="125"/>
     </row>
     <row r="65" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A65" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="B65" s="125" t="s">
+      <c r="B65" s="124" t="s">
         <v>513</v>
       </c>
-      <c r="C65" s="126"/>
-      <c r="D65" s="126"/>
-      <c r="E65" s="126"/>
+      <c r="C65" s="125"/>
+      <c r="D65" s="125"/>
+      <c r="E65" s="125"/>
     </row>
     <row r="66" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A66" s="1" t="s">
@@ -9445,23 +9457,23 @@
       <c r="A72" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="B72" s="125" t="s">
+      <c r="B72" s="124" t="s">
         <v>519</v>
       </c>
-      <c r="C72" s="126"/>
-      <c r="D72" s="126"/>
-      <c r="E72" s="126"/>
+      <c r="C72" s="125"/>
+      <c r="D72" s="125"/>
+      <c r="E72" s="125"/>
     </row>
     <row r="73" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A73" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="B73" s="125" t="s">
+      <c r="B73" s="124" t="s">
         <v>520</v>
       </c>
-      <c r="C73" s="126"/>
-      <c r="D73" s="126"/>
-      <c r="E73" s="126"/>
+      <c r="C73" s="125"/>
+      <c r="D73" s="125"/>
+      <c r="E73" s="125"/>
     </row>
     <row r="74" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A74" s="1" t="s">
@@ -9515,23 +9527,23 @@
       <c r="A78" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="B78" s="125" t="s">
+      <c r="B78" s="124" t="s">
         <v>525</v>
       </c>
-      <c r="C78" s="126"/>
-      <c r="D78" s="126"/>
-      <c r="E78" s="126"/>
+      <c r="C78" s="125"/>
+      <c r="D78" s="125"/>
+      <c r="E78" s="125"/>
     </row>
     <row r="79" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A79" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="B79" s="125" t="s">
+      <c r="B79" s="124" t="s">
         <v>526</v>
       </c>
-      <c r="C79" s="126"/>
-      <c r="D79" s="126"/>
-      <c r="E79" s="126"/>
+      <c r="C79" s="125"/>
+      <c r="D79" s="125"/>
+      <c r="E79" s="125"/>
     </row>
     <row r="80" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A80" s="1" t="s">
@@ -9643,23 +9655,23 @@
       <c r="A89" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="B89" s="125" t="s">
+      <c r="B89" s="124" t="s">
         <v>538</v>
       </c>
-      <c r="C89" s="126"/>
-      <c r="D89" s="126"/>
-      <c r="E89" s="126"/>
+      <c r="C89" s="125"/>
+      <c r="D89" s="125"/>
+      <c r="E89" s="125"/>
     </row>
     <row r="90" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A90" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="B90" s="125" t="s">
+      <c r="B90" s="124" t="s">
         <v>539</v>
       </c>
-      <c r="C90" s="126"/>
-      <c r="D90" s="126"/>
-      <c r="E90" s="126"/>
+      <c r="C90" s="125"/>
+      <c r="D90" s="125"/>
+      <c r="E90" s="125"/>
     </row>
     <row r="91" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A91" s="1" t="s">
@@ -9741,23 +9753,23 @@
       <c r="A97" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="B97" s="125" t="s">
+      <c r="B97" s="124" t="s">
         <v>548</v>
       </c>
-      <c r="C97" s="126"/>
-      <c r="D97" s="126"/>
-      <c r="E97" s="126"/>
+      <c r="C97" s="125"/>
+      <c r="D97" s="125"/>
+      <c r="E97" s="125"/>
     </row>
     <row r="98" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A98" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="B98" s="125" t="s">
+      <c r="B98" s="124" t="s">
         <v>549</v>
       </c>
-      <c r="C98" s="126"/>
-      <c r="D98" s="126"/>
-      <c r="E98" s="126"/>
+      <c r="C98" s="125"/>
+      <c r="D98" s="125"/>
+      <c r="E98" s="125"/>
     </row>
     <row r="99" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A99" s="1" t="s">
@@ -9864,23 +9876,23 @@
       <c r="A107" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="B107" s="125" t="s">
+      <c r="B107" s="124" t="s">
         <v>555</v>
       </c>
-      <c r="C107" s="126"/>
-      <c r="D107" s="126"/>
-      <c r="E107" s="126"/>
+      <c r="C107" s="125"/>
+      <c r="D107" s="125"/>
+      <c r="E107" s="125"/>
     </row>
     <row r="108" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A108" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="B108" s="125" t="s">
+      <c r="B108" s="124" t="s">
         <v>556</v>
       </c>
-      <c r="C108" s="126"/>
-      <c r="D108" s="126"/>
-      <c r="E108" s="126"/>
+      <c r="C108" s="125"/>
+      <c r="D108" s="125"/>
+      <c r="E108" s="125"/>
     </row>
     <row r="109" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A109" s="1" t="s">
@@ -9956,23 +9968,23 @@
       <c r="A115" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="B115" s="125" t="s">
+      <c r="B115" s="124" t="s">
         <v>563</v>
       </c>
-      <c r="C115" s="126"/>
-      <c r="D115" s="126"/>
-      <c r="E115" s="126"/>
+      <c r="C115" s="125"/>
+      <c r="D115" s="125"/>
+      <c r="E115" s="125"/>
     </row>
     <row r="116" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A116" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="B116" s="125" t="s">
+      <c r="B116" s="124" t="s">
         <v>564</v>
       </c>
-      <c r="C116" s="126"/>
-      <c r="D116" s="126"/>
-      <c r="E116" s="126"/>
+      <c r="C116" s="125"/>
+      <c r="D116" s="125"/>
+      <c r="E116" s="125"/>
     </row>
     <row r="117" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A117" s="1" t="s">
@@ -10062,23 +10074,23 @@
       <c r="A124" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="B124" s="125" t="s">
+      <c r="B124" s="124" t="s">
         <v>572</v>
       </c>
-      <c r="C124" s="126"/>
-      <c r="D124" s="126"/>
-      <c r="E124" s="126"/>
+      <c r="C124" s="125"/>
+      <c r="D124" s="125"/>
+      <c r="E124" s="125"/>
     </row>
     <row r="125" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A125" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="B125" s="125" t="s">
+      <c r="B125" s="124" t="s">
         <v>573</v>
       </c>
-      <c r="C125" s="126"/>
-      <c r="D125" s="126"/>
-      <c r="E125" s="126"/>
+      <c r="C125" s="125"/>
+      <c r="D125" s="125"/>
+      <c r="E125" s="125"/>
     </row>
     <row r="126" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A126" s="1" t="s">
@@ -10165,23 +10177,23 @@
       <c r="A133" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="B133" s="125" t="s">
+      <c r="B133" s="124" t="s">
         <v>580</v>
       </c>
-      <c r="C133" s="126"/>
-      <c r="D133" s="126"/>
-      <c r="E133" s="126"/>
+      <c r="C133" s="125"/>
+      <c r="D133" s="125"/>
+      <c r="E133" s="125"/>
     </row>
     <row r="134" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A134" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="B134" s="125" t="s">
+      <c r="B134" s="124" t="s">
         <v>581</v>
       </c>
-      <c r="C134" s="126"/>
-      <c r="D134" s="126"/>
-      <c r="E134" s="126"/>
+      <c r="C134" s="125"/>
+      <c r="D134" s="125"/>
+      <c r="E134" s="125"/>
     </row>
     <row r="135" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A135" s="1" t="s">
@@ -10333,39 +10345,39 @@
     </row>
   </sheetData>
   <mergeCells count="33">
-    <mergeCell ref="B116:E116"/>
-    <mergeCell ref="B124:E124"/>
-    <mergeCell ref="B125:E125"/>
-    <mergeCell ref="B133:E133"/>
-    <mergeCell ref="B134:E134"/>
-    <mergeCell ref="B97:E97"/>
-    <mergeCell ref="B98:E98"/>
-    <mergeCell ref="B107:E107"/>
-    <mergeCell ref="B108:E108"/>
-    <mergeCell ref="B115:E115"/>
-    <mergeCell ref="B3:E3"/>
-    <mergeCell ref="B4:E4"/>
-    <mergeCell ref="B33:E33"/>
-    <mergeCell ref="B39:E39"/>
-    <mergeCell ref="B45:E45"/>
-    <mergeCell ref="A1:E1"/>
-    <mergeCell ref="B38:E38"/>
-    <mergeCell ref="B24:E24"/>
-    <mergeCell ref="B23:E23"/>
-    <mergeCell ref="B32:E32"/>
-    <mergeCell ref="B44:E44"/>
+    <mergeCell ref="B90:E90"/>
+    <mergeCell ref="B79:E79"/>
+    <mergeCell ref="B58:E58"/>
+    <mergeCell ref="B64:E64"/>
+    <mergeCell ref="B65:E65"/>
+    <mergeCell ref="B89:E89"/>
     <mergeCell ref="B50:E50"/>
     <mergeCell ref="B51:E51"/>
     <mergeCell ref="B78:E78"/>
     <mergeCell ref="B59:E59"/>
     <mergeCell ref="B72:E72"/>
     <mergeCell ref="B73:E73"/>
-    <mergeCell ref="B79:E79"/>
-    <mergeCell ref="B58:E58"/>
-    <mergeCell ref="B64:E64"/>
-    <mergeCell ref="B65:E65"/>
-    <mergeCell ref="B89:E89"/>
-    <mergeCell ref="B90:E90"/>
+    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="B38:E38"/>
+    <mergeCell ref="B24:E24"/>
+    <mergeCell ref="B23:E23"/>
+    <mergeCell ref="B32:E32"/>
+    <mergeCell ref="B3:E3"/>
+    <mergeCell ref="B4:E4"/>
+    <mergeCell ref="B33:E33"/>
+    <mergeCell ref="B39:E39"/>
+    <mergeCell ref="B45:E45"/>
+    <mergeCell ref="B44:E44"/>
+    <mergeCell ref="B97:E97"/>
+    <mergeCell ref="B98:E98"/>
+    <mergeCell ref="B107:E107"/>
+    <mergeCell ref="B108:E108"/>
+    <mergeCell ref="B115:E115"/>
+    <mergeCell ref="B116:E116"/>
+    <mergeCell ref="B124:E124"/>
+    <mergeCell ref="B125:E125"/>
+    <mergeCell ref="B133:E133"/>
+    <mergeCell ref="B134:E134"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -10796,14 +10808,14 @@
       </c>
     </row>
     <row r="9" spans="1:20" ht="29.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="I9" s="124" t="s">
+      <c r="I9" s="86" t="s">
         <v>217</v>
       </c>
-      <c r="J9" s="124"/>
-      <c r="K9" s="124"/>
-      <c r="L9" s="124"/>
-      <c r="M9" s="124"/>
-      <c r="N9" s="124"/>
+      <c r="J9" s="86"/>
+      <c r="K9" s="86"/>
+      <c r="L9" s="86"/>
+      <c r="M9" s="86"/>
+      <c r="N9" s="86"/>
     </row>
     <row r="11" spans="1:20" ht="15.75" x14ac:dyDescent="0.25">
       <c r="I11" s="21" t="s">
@@ -10865,4 +10877,10 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
+<clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
+  <clbl:label id="{d1b36e95-0d50-42e9-958f-b63fa906beaa}" enabled="0" method="" siteId="{d1b36e95-0d50-42e9-958f-b63fa906beaa}" removed="1"/>
+</clbl:labelList>
 </file>
</xml_diff>

<commit_message>
Added agent password risk
</commit_message>
<xml_diff>
--- a/docs/Datathon Project.xlsx
+++ b/docs/Datathon Project.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Anchit\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://uoa-my.sharepoint.com/personal/ghin287_uoa_auckland_ac_nz/Documents/Documents/University/Datathon temp/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3D3FBC14-72BA-42A7-A028-E7A78C040042}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{B1F4A7BC-5C27-4579-8900-F0D73B159D0E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" activeTab="1" xr2:uid="{B8873715-DDF3-4B00-844B-82E399C3542D}"/>
+    <workbookView xWindow="7536" yWindow="17172" windowWidth="23256" windowHeight="12456" activeTab="4" xr2:uid="{B8873715-DDF3-4B00-844B-82E399C3542D}"/>
   </bookViews>
   <sheets>
     <sheet name="Team Overview" sheetId="2" r:id="rId1"/>
@@ -28,7 +28,7 @@
     <externalReference r:id="rId11"/>
   </externalReferences>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'RAID Logs '!$A$1:$M$37</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'RAID Logs '!$A$1:$M$38</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -49,7 +49,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1204" uniqueCount="588">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1210" uniqueCount="591">
   <si>
     <t>court</t>
   </si>
@@ -2049,6 +2049,15 @@
   <si>
     <t>6 gramss- Team 4</t>
   </si>
+  <si>
+    <t>R09</t>
+  </si>
+  <si>
+    <t>Hardcoded password in git history in 003_CreateIngestionAgentRoles.sql</t>
+  </si>
+  <si>
+    <t>file provided in github for marking purposes, but would be correctly held in Snowflake and run via python script from .env. Low immediate risk for POC.</t>
+  </si>
 </sst>
 </file>
 
@@ -2057,7 +2066,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="dd\ mmm\ yyyy"/>
   </numFmts>
-  <fonts count="27">
+  <fonts count="27" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -2831,6 +2840,21 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="15" fontId="0" fillId="17" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="19" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="3" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -2845,21 +2869,6 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="3" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -2933,6 +2942,9 @@
     <xf numFmtId="0" fontId="15" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -2947,9 +2959,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -2984,34 +2993,6 @@
       <fill>
         <patternFill>
           <bgColor rgb="FF92D050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="5" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="8" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFCCCC"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.59996337778862885"/>
         </patternFill>
       </fill>
     </dxf>
@@ -3075,6 +3056,34 @@
       <fill>
         <patternFill>
           <bgColor rgb="FFF4B6B6"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="5" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="8" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFCCCC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.59996337778862885"/>
         </patternFill>
       </fill>
     </dxf>
@@ -3932,7 +3941,7 @@
 </file>
 
 <file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" mc:Ignorable="x14">
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
     <sheetNames>
       <sheetName val="Summary"/>
@@ -4348,9 +4357,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -4388,7 +4397,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -4494,7 +4503,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -4636,7 +4645,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -4645,103 +4654,103 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{70241A6B-2CF1-42DB-9288-7E14FFCD0A5F}">
   <dimension ref="A1:G36"/>
-  <sheetFormatPr defaultColWidth="21.26953125" defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultColWidth="21.28515625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="25.453125" customWidth="1"/>
-    <col min="2" max="2" width="73.54296875" customWidth="1"/>
+    <col min="1" max="1" width="25.42578125" customWidth="1"/>
+    <col min="2" max="2" width="73.5703125" customWidth="1"/>
     <col min="4" max="4" width="70" customWidth="1"/>
-    <col min="5" max="5" width="49.81640625" customWidth="1"/>
-    <col min="6" max="6" width="28.54296875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="49.85546875" customWidth="1"/>
+    <col min="6" max="6" width="28.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="54.65" customHeight="1">
-      <c r="A1" s="89" t="s">
+    <row r="1" spans="1:7" ht="54.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="94" t="s">
         <v>263</v>
       </c>
-      <c r="B1" s="90"/>
-      <c r="C1" s="90"/>
-      <c r="D1" s="90"/>
-      <c r="E1" s="90"/>
-      <c r="F1" s="90"/>
-    </row>
-    <row r="3" spans="1:7">
+      <c r="B1" s="95"/>
+      <c r="C1" s="95"/>
+      <c r="D1" s="95"/>
+      <c r="E1" s="95"/>
+      <c r="F1" s="95"/>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="39" t="s">
         <v>78</v>
       </c>
       <c r="B3" s="37" t="s">
         <v>84</v>
       </c>
-      <c r="D3" s="89" t="s">
+      <c r="D3" s="94" t="s">
         <v>587</v>
       </c>
-      <c r="E3" s="90"/>
+      <c r="E3" s="95"/>
       <c r="F3" s="3"/>
       <c r="G3" s="7" t="s">
         <v>86</v>
       </c>
     </row>
-    <row r="4" spans="1:7">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="39" t="s">
         <v>75</v>
       </c>
       <c r="B4" s="40" t="s">
         <v>77</v>
       </c>
-      <c r="D4" s="89"/>
-      <c r="E4" s="90"/>
+      <c r="D4" s="94"/>
+      <c r="E4" s="95"/>
       <c r="F4" s="3"/>
       <c r="G4" s="12" t="s">
         <v>85</v>
       </c>
     </row>
-    <row r="5" spans="1:7">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="39" t="s">
         <v>76</v>
       </c>
       <c r="B5" s="40" t="s">
         <v>312</v>
       </c>
-      <c r="D5" s="89"/>
-      <c r="E5" s="90"/>
+      <c r="D5" s="94"/>
+      <c r="E5" s="95"/>
       <c r="F5" s="3"/>
       <c r="G5" s="11" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="6" spans="1:7">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="39" t="s">
         <v>68</v>
       </c>
       <c r="B6" s="37" t="s">
         <v>87</v>
       </c>
-      <c r="D6" s="89"/>
-      <c r="E6" s="90"/>
+      <c r="D6" s="94"/>
+      <c r="E6" s="95"/>
       <c r="F6" s="3"/>
       <c r="G6" s="10" t="s">
         <v>88</v>
       </c>
     </row>
-    <row r="7" spans="1:7">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="50"/>
       <c r="B7" s="51"/>
-      <c r="D7" s="89"/>
-      <c r="E7" s="90"/>
+      <c r="D7" s="94"/>
+      <c r="E7" s="95"/>
       <c r="F7" s="3"/>
     </row>
-    <row r="10" spans="1:7" ht="62.5" customHeight="1">
-      <c r="A10" s="88" t="s">
+    <row r="10" spans="1:7" ht="62.45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="93" t="s">
         <v>290</v>
       </c>
-      <c r="B10" s="88"/>
-      <c r="C10" s="88"/>
-      <c r="D10" s="88" t="s">
+      <c r="B10" s="93"/>
+      <c r="C10" s="93"/>
+      <c r="D10" s="93" t="s">
         <v>291</v>
       </c>
-      <c r="E10" s="88"/>
-      <c r="F10" s="88"/>
-    </row>
-    <row r="11" spans="1:7" ht="27" customHeight="1">
+      <c r="E10" s="93"/>
+      <c r="F10" s="93"/>
+    </row>
+    <row r="11" spans="1:7" ht="27" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="56" t="s">
         <v>18</v>
       </c>
@@ -4761,7 +4770,7 @@
         <v>286</v>
       </c>
     </row>
-    <row r="12" spans="1:7" ht="43.5">
+    <row r="12" spans="1:7" ht="45" x14ac:dyDescent="0.25">
       <c r="A12" s="52" t="s">
         <v>8</v>
       </c>
@@ -4781,7 +4790,7 @@
         <v>264</v>
       </c>
     </row>
-    <row r="13" spans="1:7" ht="72.5">
+    <row r="13" spans="1:7" ht="75" x14ac:dyDescent="0.25">
       <c r="A13" s="32" t="s">
         <v>9</v>
       </c>
@@ -4801,7 +4810,7 @@
         <v>272</v>
       </c>
     </row>
-    <row r="14" spans="1:7" ht="43.5">
+    <row r="14" spans="1:7" ht="45" x14ac:dyDescent="0.25">
       <c r="A14" s="32" t="s">
         <v>6</v>
       </c>
@@ -4821,7 +4830,7 @@
         <v>268</v>
       </c>
     </row>
-    <row r="15" spans="1:7" ht="29">
+    <row r="15" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A15" s="32" t="s">
         <v>7</v>
       </c>
@@ -4841,7 +4850,7 @@
         <v>267</v>
       </c>
     </row>
-    <row r="16" spans="1:7">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" s="32" t="s">
         <v>4</v>
       </c>
@@ -4859,7 +4868,7 @@
         <v>265</v>
       </c>
     </row>
-    <row r="17" spans="1:6">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17" s="32" t="s">
         <v>5</v>
       </c>
@@ -4879,13 +4888,13 @@
         <v>315</v>
       </c>
     </row>
-    <row r="20" spans="1:6">
-      <c r="A20" s="86" t="s">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A20" s="91" t="s">
         <v>258</v>
       </c>
-      <c r="B20" s="87"/>
-    </row>
-    <row r="21" spans="1:6" ht="22.5" customHeight="1">
+      <c r="B20" s="92"/>
+    </row>
+    <row r="21" spans="1:6" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="57" t="s">
         <v>18</v>
       </c>
@@ -4893,7 +4902,7 @@
         <v>259</v>
       </c>
     </row>
-    <row r="22" spans="1:6" ht="29">
+    <row r="22" spans="1:6" ht="45" x14ac:dyDescent="0.25">
       <c r="A22" s="79" t="s">
         <v>289</v>
       </c>
@@ -4901,7 +4910,7 @@
         <v>262</v>
       </c>
     </row>
-    <row r="23" spans="1:6">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A23" s="78" t="s">
         <v>260</v>
       </c>
@@ -4909,7 +4918,7 @@
         <v>261</v>
       </c>
     </row>
-    <row r="24" spans="1:6">
+    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A24" s="78" t="s">
         <v>79</v>
       </c>
@@ -4917,7 +4926,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="25" spans="1:6">
+    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A25" s="32" t="s">
         <v>90</v>
       </c>
@@ -4925,7 +4934,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="26" spans="1:6">
+    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A26" s="32" t="s">
         <v>89</v>
       </c>
@@ -4933,7 +4942,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="27" spans="1:6">
+    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A27" s="32" t="s">
         <v>91</v>
       </c>
@@ -4941,7 +4950,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="28" spans="1:6">
+    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A28" s="32" t="s">
         <v>288</v>
       </c>
@@ -4949,7 +4958,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="31" spans="1:6">
+    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A31" s="80" t="s">
         <v>70</v>
       </c>
@@ -4957,7 +4966,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="32" spans="1:6">
+    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A32" s="81" t="s">
         <v>311</v>
       </c>
@@ -4965,7 +4974,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="33" spans="1:2">
+    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A33" s="81" t="s">
         <v>73</v>
       </c>
@@ -4973,7 +4982,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="34" spans="1:2">
+    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A34" s="81" t="s">
         <v>313</v>
       </c>
@@ -4981,7 +4990,7 @@
         <v>314</v>
       </c>
     </row>
-    <row r="36" spans="1:2" ht="14.5" customHeight="1"/>
+    <row r="36" spans="1:2" ht="14.45" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="5">
     <mergeCell ref="A20:B20"/>
@@ -5059,18 +5068,18 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C3DCDC7C-55B3-416C-9E03-05A0A063B246}">
   <dimension ref="A1:N9"/>
-  <sheetFormatPr defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="18.81640625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="4.453125" customWidth="1"/>
+    <col min="10" max="10" width="18.85546875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="4.42578125" customWidth="1"/>
     <col min="12" max="12" width="14" customWidth="1"/>
-    <col min="13" max="13" width="6.1796875" customWidth="1"/>
-    <col min="14" max="14" width="11.81640625" customWidth="1"/>
-    <col min="17" max="17" width="18.81640625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="6.140625" customWidth="1"/>
+    <col min="14" max="14" width="11.85546875" customWidth="1"/>
+    <col min="17" max="17" width="18.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14">
+    <row r="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1" s="27" t="s">
         <v>29</v>
       </c>
@@ -5102,7 +5111,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="2" spans="1:14">
+    <row r="2" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A2" s="42" t="s">
         <v>0</v>
       </c>
@@ -5132,7 +5141,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="3" spans="1:14">
+    <row r="3" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A3" s="42" t="s">
         <v>1</v>
       </c>
@@ -5156,7 +5165,7 @@
         <v>273</v>
       </c>
     </row>
-    <row r="4" spans="1:14">
+    <row r="4" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A4" s="42" t="s">
         <v>2</v>
       </c>
@@ -5180,7 +5189,7 @@
         <v>281</v>
       </c>
     </row>
-    <row r="5" spans="1:14">
+    <row r="5" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A5" s="42" t="s">
         <v>3</v>
       </c>
@@ -5206,7 +5215,7 @@
         <v>276</v>
       </c>
     </row>
-    <row r="9" spans="1:14" ht="29.15" customHeight="1"/>
+    <row r="9" spans="1:14" ht="29.1" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -5216,21 +5225,21 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DB583F5E-2C32-4E7A-802B-32AB9008611B}">
   <dimension ref="A1:I35"/>
-  <sheetFormatPr defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="8.453125" customWidth="1"/>
-    <col min="2" max="2" width="110.54296875" customWidth="1"/>
-    <col min="3" max="3" width="20.54296875" style="4" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="15.453125" style="4" customWidth="1"/>
-    <col min="6" max="6" width="28.1796875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="29.54296875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="27.453125" customWidth="1"/>
+    <col min="1" max="1" width="8.42578125" customWidth="1"/>
+    <col min="2" max="2" width="110.5703125" customWidth="1"/>
+    <col min="3" max="3" width="20.5703125" style="4" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15.42578125" style="4" customWidth="1"/>
+    <col min="6" max="6" width="28.140625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="29.5703125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="27.42578125" customWidth="1"/>
     <col min="9" max="9" width="51" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="5.54296875" customWidth="1"/>
-    <col min="11" max="11" width="8.1796875" customWidth="1"/>
+    <col min="10" max="10" width="5.5703125" customWidth="1"/>
+    <col min="11" max="11" width="8.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="43" customHeight="1">
+    <row r="1" spans="1:9" ht="42.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="28" t="s">
         <v>277</v>
       </c>
@@ -5254,7 +5263,7 @@
         <v>230</v>
       </c>
     </row>
-    <row r="2" spans="1:9" ht="43.5">
+    <row r="2" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A2" s="32">
         <v>1</v>
       </c>
@@ -5277,7 +5286,7 @@
         <v>233</v>
       </c>
     </row>
-    <row r="3" spans="1:9" ht="29">
+    <row r="3" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A3" s="32">
         <v>2</v>
       </c>
@@ -5300,7 +5309,7 @@
         <v>233</v>
       </c>
     </row>
-    <row r="4" spans="1:9" ht="29">
+    <row r="4" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A4" s="32">
         <v>3</v>
       </c>
@@ -5323,7 +5332,7 @@
         <v>233</v>
       </c>
     </row>
-    <row r="5" spans="1:9" ht="29">
+    <row r="5" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A5" s="32">
         <v>4</v>
       </c>
@@ -5346,7 +5355,7 @@
         <v>241</v>
       </c>
     </row>
-    <row r="6" spans="1:9">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" s="32">
         <v>5</v>
       </c>
@@ -5369,7 +5378,7 @@
         <v>241</v>
       </c>
     </row>
-    <row r="7" spans="1:9" ht="29">
+    <row r="7" spans="1:9" ht="30.75" x14ac:dyDescent="0.25">
       <c r="A7" s="32">
         <v>6</v>
       </c>
@@ -5392,7 +5401,7 @@
         <v>247</v>
       </c>
     </row>
-    <row r="8" spans="1:9" ht="87">
+    <row r="8" spans="1:9" ht="90" x14ac:dyDescent="0.25">
       <c r="A8" s="32">
         <v>7</v>
       </c>
@@ -5403,7 +5412,7 @@
         <v>281</v>
       </c>
     </row>
-    <row r="9" spans="1:9" ht="72.5">
+    <row r="9" spans="1:9" ht="75" x14ac:dyDescent="0.25">
       <c r="A9" s="32">
         <v>8</v>
       </c>
@@ -5413,14 +5422,14 @@
       <c r="C9" s="32" t="s">
         <v>34</v>
       </c>
-      <c r="F9" s="91" t="s">
+      <c r="F9" s="86" t="s">
         <v>308</v>
       </c>
-      <c r="G9" s="92"/>
-      <c r="H9" s="92"/>
-      <c r="I9" s="93"/>
-    </row>
-    <row r="10" spans="1:9">
+      <c r="G9" s="87"/>
+      <c r="H9" s="87"/>
+      <c r="I9" s="88"/>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10" s="32">
         <v>9</v>
       </c>
@@ -5431,7 +5440,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="11" spans="1:9">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11" s="32">
         <v>10</v>
       </c>
@@ -5442,7 +5451,7 @@
         <v>276</v>
       </c>
     </row>
-    <row r="12" spans="1:9">
+    <row r="12" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A12" s="32">
         <v>11</v>
       </c>
@@ -5453,81 +5462,81 @@
         <v>273</v>
       </c>
     </row>
-    <row r="14" spans="1:9" ht="14.5" customHeight="1">
-      <c r="B14" s="94" t="s">
+    <row r="14" spans="1:9" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B14" s="89" t="s">
         <v>326</v>
       </c>
-      <c r="C14" s="94"/>
-    </row>
-    <row r="15" spans="1:9">
-      <c r="B15" s="94"/>
-      <c r="C15" s="94"/>
-    </row>
-    <row r="16" spans="1:9">
-      <c r="B16" s="94"/>
-      <c r="C16" s="94"/>
-    </row>
-    <row r="17" spans="2:3">
-      <c r="B17" s="94"/>
-      <c r="C17" s="94"/>
-    </row>
-    <row r="18" spans="2:3">
-      <c r="B18" s="94"/>
-      <c r="C18" s="94"/>
-    </row>
-    <row r="19" spans="2:3">
-      <c r="B19" s="94"/>
-      <c r="C19" s="94"/>
-    </row>
-    <row r="20" spans="2:3">
-      <c r="B20" s="94"/>
-      <c r="C20" s="94"/>
-    </row>
-    <row r="21" spans="2:3">
-      <c r="B21" s="94"/>
-      <c r="C21" s="94"/>
-    </row>
-    <row r="22" spans="2:3">
-      <c r="B22" s="94"/>
-      <c r="C22" s="94"/>
-    </row>
-    <row r="23" spans="2:3">
-      <c r="B23" s="94"/>
-      <c r="C23" s="94"/>
-    </row>
-    <row r="24" spans="2:3">
-      <c r="B24" s="94"/>
-      <c r="C24" s="94"/>
-    </row>
-    <row r="26" spans="2:3" ht="14.5" customHeight="1"/>
-    <row r="27" spans="2:3">
+      <c r="C14" s="89"/>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="B15" s="89"/>
+      <c r="C15" s="89"/>
+    </row>
+    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="B16" s="89"/>
+      <c r="C16" s="89"/>
+    </row>
+    <row r="17" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B17" s="89"/>
+      <c r="C17" s="89"/>
+    </row>
+    <row r="18" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B18" s="89"/>
+      <c r="C18" s="89"/>
+    </row>
+    <row r="19" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B19" s="89"/>
+      <c r="C19" s="89"/>
+    </row>
+    <row r="20" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B20" s="89"/>
+      <c r="C20" s="89"/>
+    </row>
+    <row r="21" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B21" s="89"/>
+      <c r="C21" s="89"/>
+    </row>
+    <row r="22" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B22" s="89"/>
+      <c r="C22" s="89"/>
+    </row>
+    <row r="23" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B23" s="89"/>
+      <c r="C23" s="89"/>
+    </row>
+    <row r="24" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B24" s="89"/>
+      <c r="C24" s="89"/>
+    </row>
+    <row r="26" spans="2:3" ht="14.45" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="27" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B27" s="3"/>
     </row>
-    <row r="28" spans="2:3" ht="72.650000000000006" customHeight="1">
-      <c r="B28" s="95" t="s">
+    <row r="28" spans="2:3" ht="72.599999999999994" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B28" s="90" t="s">
         <v>327</v>
       </c>
-      <c r="C28" s="95"/>
-    </row>
-    <row r="29" spans="2:3">
+      <c r="C28" s="90"/>
+    </row>
+    <row r="29" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B29" s="3"/>
     </row>
-    <row r="30" spans="2:3">
+    <row r="30" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B30" s="3"/>
     </row>
-    <row r="31" spans="2:3">
+    <row r="31" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B31" s="3"/>
     </row>
-    <row r="32" spans="2:3">
+    <row r="32" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B32" s="3"/>
     </row>
-    <row r="33" spans="2:2">
+    <row r="33" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B33" s="3"/>
     </row>
-    <row r="34" spans="2:2">
+    <row r="34" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B34" s="3"/>
     </row>
-    <row r="35" spans="2:2">
+    <row r="35" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B35" s="3"/>
     </row>
   </sheetData>
@@ -5557,17 +5566,17 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AA72A998-9D73-4F3B-A55F-A4F70ED3DBFB}">
   <dimension ref="B1:J30"/>
-  <sheetFormatPr defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="2.1796875" customWidth="1"/>
-    <col min="2" max="2" width="44.453125" style="3" customWidth="1"/>
-    <col min="3" max="3" width="39.1796875" customWidth="1"/>
-    <col min="4" max="4" width="17.7265625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="11.54296875" customWidth="1"/>
-    <col min="6" max="6" width="23.81640625" hidden="1" customWidth="1"/>
+    <col min="1" max="1" width="2.140625" customWidth="1"/>
+    <col min="2" max="2" width="44.42578125" style="3" customWidth="1"/>
+    <col min="3" max="3" width="39.140625" customWidth="1"/>
+    <col min="4" max="4" width="17.7109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11.5703125" customWidth="1"/>
+    <col min="6" max="6" width="23.85546875" hidden="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:10" ht="30.65" customHeight="1">
+    <row r="1" spans="2:10" ht="30.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B1" s="26" t="s">
         <v>107</v>
       </c>
@@ -5579,7 +5588,7 @@
       </c>
       <c r="E1" s="2"/>
     </row>
-    <row r="2" spans="2:10" ht="29.15" customHeight="1">
+    <row r="2" spans="2:10" ht="29.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B2" s="36" t="s">
         <v>227</v>
       </c>
@@ -5596,7 +5605,7 @@
       <c r="I2" s="98"/>
       <c r="J2" s="99"/>
     </row>
-    <row r="3" spans="2:10" ht="14.5" customHeight="1">
+    <row r="3" spans="2:10" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B3" s="36" t="s">
         <v>100</v>
       </c>
@@ -5611,7 +5620,7 @@
       <c r="I3" s="101"/>
       <c r="J3" s="102"/>
     </row>
-    <row r="4" spans="2:10" ht="14.5" customHeight="1">
+    <row r="4" spans="2:10" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B4" s="36" t="s">
         <v>317</v>
       </c>
@@ -5626,7 +5635,7 @@
       <c r="I4" s="101"/>
       <c r="J4" s="102"/>
     </row>
-    <row r="5" spans="2:10" ht="14.5" customHeight="1">
+    <row r="5" spans="2:10" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B5" s="36" t="s">
         <v>104</v>
       </c>
@@ -5641,7 +5650,7 @@
       <c r="I5" s="104"/>
       <c r="J5" s="105"/>
     </row>
-    <row r="6" spans="2:10" ht="29">
+    <row r="6" spans="2:10" ht="30" x14ac:dyDescent="0.25">
       <c r="B6" s="36" t="s">
         <v>318</v>
       </c>
@@ -5652,7 +5661,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="7" spans="2:10">
+    <row r="7" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B7" s="36" t="s">
         <v>105</v>
       </c>
@@ -5663,7 +5672,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="8" spans="2:10" ht="14.5" customHeight="1">
+    <row r="8" spans="2:10" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B8" s="36" t="s">
         <v>422</v>
       </c>
@@ -5680,7 +5689,7 @@
       <c r="I8" s="107"/>
       <c r="J8" s="108"/>
     </row>
-    <row r="9" spans="2:10">
+    <row r="9" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B9" s="36" t="s">
         <v>99</v>
       </c>
@@ -5695,7 +5704,7 @@
       <c r="I9" s="110"/>
       <c r="J9" s="111"/>
     </row>
-    <row r="10" spans="2:10" ht="14.5" customHeight="1">
+    <row r="10" spans="2:10" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B10" s="36" t="s">
         <v>252</v>
       </c>
@@ -5710,73 +5719,73 @@
       <c r="I10" s="110"/>
       <c r="J10" s="111"/>
     </row>
-    <row r="11" spans="2:10">
+    <row r="11" spans="2:10" x14ac:dyDescent="0.25">
       <c r="G11" s="109"/>
       <c r="H11" s="110"/>
       <c r="I11" s="110"/>
       <c r="J11" s="111"/>
     </row>
-    <row r="12" spans="2:10" ht="14.5" customHeight="1">
+    <row r="12" spans="2:10" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="G12" s="112"/>
       <c r="H12" s="113"/>
       <c r="I12" s="113"/>
       <c r="J12" s="114"/>
     </row>
-    <row r="13" spans="2:10" ht="14.5" customHeight="1"/>
-    <row r="14" spans="2:10" ht="14.5" customHeight="1">
-      <c r="G14" s="94" t="s">
+    <row r="13" spans="2:10" ht="14.45" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="14" spans="2:10" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G14" s="89" t="s">
         <v>249</v>
       </c>
-      <c r="H14" s="94"/>
-      <c r="I14" s="94"/>
-      <c r="J14" s="94"/>
-    </row>
-    <row r="15" spans="2:10">
-      <c r="G15" s="94"/>
-      <c r="H15" s="94"/>
-      <c r="I15" s="94"/>
-      <c r="J15" s="94"/>
-    </row>
-    <row r="16" spans="2:10" ht="14.5" customHeight="1">
-      <c r="G16" s="94"/>
-      <c r="H16" s="94"/>
-      <c r="I16" s="94"/>
-      <c r="J16" s="94"/>
-    </row>
-    <row r="17" spans="7:10" ht="14.5" customHeight="1">
-      <c r="G17" s="94"/>
-      <c r="H17" s="94"/>
-      <c r="I17" s="94"/>
-      <c r="J17" s="94"/>
-    </row>
-    <row r="18" spans="7:10" ht="14.5" customHeight="1"/>
-    <row r="19" spans="7:10" ht="14.5" customHeight="1">
-      <c r="G19" s="94" t="s">
+      <c r="H14" s="89"/>
+      <c r="I14" s="89"/>
+      <c r="J14" s="89"/>
+    </row>
+    <row r="15" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="G15" s="89"/>
+      <c r="H15" s="89"/>
+      <c r="I15" s="89"/>
+      <c r="J15" s="89"/>
+    </row>
+    <row r="16" spans="2:10" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G16" s="89"/>
+      <c r="H16" s="89"/>
+      <c r="I16" s="89"/>
+      <c r="J16" s="89"/>
+    </row>
+    <row r="17" spans="7:10" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G17" s="89"/>
+      <c r="H17" s="89"/>
+      <c r="I17" s="89"/>
+      <c r="J17" s="89"/>
+    </row>
+    <row r="18" spans="7:10" ht="14.45" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="19" spans="7:10" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G19" s="89" t="s">
         <v>250</v>
       </c>
-      <c r="H19" s="94"/>
-      <c r="I19" s="94"/>
-      <c r="J19" s="94"/>
-    </row>
-    <row r="20" spans="7:10">
-      <c r="G20" s="94"/>
-      <c r="H20" s="94"/>
-      <c r="I20" s="94"/>
-      <c r="J20" s="94"/>
-    </row>
-    <row r="21" spans="7:10">
-      <c r="G21" s="94"/>
-      <c r="H21" s="94"/>
-      <c r="I21" s="94"/>
-      <c r="J21" s="94"/>
-    </row>
-    <row r="22" spans="7:10" ht="14.5" customHeight="1">
-      <c r="G22" s="94"/>
-      <c r="H22" s="94"/>
-      <c r="I22" s="94"/>
-      <c r="J22" s="94"/>
-    </row>
-    <row r="25" spans="7:10" ht="14.5" customHeight="1">
+      <c r="H19" s="89"/>
+      <c r="I19" s="89"/>
+      <c r="J19" s="89"/>
+    </row>
+    <row r="20" spans="7:10" x14ac:dyDescent="0.25">
+      <c r="G20" s="89"/>
+      <c r="H20" s="89"/>
+      <c r="I20" s="89"/>
+      <c r="J20" s="89"/>
+    </row>
+    <row r="21" spans="7:10" x14ac:dyDescent="0.25">
+      <c r="G21" s="89"/>
+      <c r="H21" s="89"/>
+      <c r="I21" s="89"/>
+      <c r="J21" s="89"/>
+    </row>
+    <row r="22" spans="7:10" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G22" s="89"/>
+      <c r="H22" s="89"/>
+      <c r="I22" s="89"/>
+      <c r="J22" s="89"/>
+    </row>
+    <row r="25" spans="7:10" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="G25" s="96" t="s">
         <v>287</v>
       </c>
@@ -5784,31 +5793,31 @@
       <c r="I25" s="96"/>
       <c r="J25" s="96"/>
     </row>
-    <row r="26" spans="7:10">
+    <row r="26" spans="7:10" x14ac:dyDescent="0.25">
       <c r="G26" s="96"/>
       <c r="H26" s="96"/>
       <c r="I26" s="96"/>
       <c r="J26" s="96"/>
     </row>
-    <row r="27" spans="7:10">
+    <row r="27" spans="7:10" x14ac:dyDescent="0.25">
       <c r="G27" s="96"/>
       <c r="H27" s="96"/>
       <c r="I27" s="96"/>
       <c r="J27" s="96"/>
     </row>
-    <row r="28" spans="7:10" ht="14.5" customHeight="1">
+    <row r="28" spans="7:10" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="G28" s="96"/>
       <c r="H28" s="96"/>
       <c r="I28" s="96"/>
       <c r="J28" s="96"/>
     </row>
-    <row r="29" spans="7:10">
+    <row r="29" spans="7:10" x14ac:dyDescent="0.25">
       <c r="G29" s="96"/>
       <c r="H29" s="96"/>
       <c r="I29" s="96"/>
       <c r="J29" s="96"/>
     </row>
-    <row r="30" spans="7:10">
+    <row r="30" spans="7:10" x14ac:dyDescent="0.25">
       <c r="G30" s="96"/>
       <c r="H30" s="96"/>
       <c r="I30" s="96"/>
@@ -5890,19 +5899,19 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BD6A8ABF-E61F-4C75-ADCE-19B4345AB4F4}">
   <dimension ref="A1:AK33"/>
-  <sheetFormatPr defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="37.54296875" customWidth="1"/>
-    <col min="2" max="2" width="35.1796875" customWidth="1"/>
-    <col min="3" max="3" width="43.54296875" customWidth="1"/>
+    <col min="1" max="1" width="37.5703125" customWidth="1"/>
+    <col min="2" max="2" width="35.140625" customWidth="1"/>
+    <col min="3" max="3" width="43.5703125" customWidth="1"/>
     <col min="6" max="6" width="23" customWidth="1"/>
-    <col min="8" max="8" width="41.1796875" customWidth="1"/>
-    <col min="35" max="35" width="42.26953125" customWidth="1"/>
-    <col min="36" max="36" width="48.453125" customWidth="1"/>
-    <col min="37" max="37" width="66.7265625" customWidth="1"/>
+    <col min="8" max="8" width="41.140625" customWidth="1"/>
+    <col min="35" max="35" width="42.28515625" customWidth="1"/>
+    <col min="36" max="36" width="48.42578125" customWidth="1"/>
+    <col min="37" max="37" width="66.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:37" ht="37.5" customHeight="1">
+    <row r="1" spans="1:37" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="118" t="s">
         <v>421</v>
       </c>
@@ -5944,7 +5953,7 @@
       <c r="AJ1" s="116"/>
       <c r="AK1" s="117"/>
     </row>
-    <row r="33" spans="1:12" ht="42.65" customHeight="1">
+    <row r="33" spans="1:12" ht="42.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="115" t="s">
         <v>329</v>
       </c>
@@ -5976,27 +5985,27 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B61A661B-79AD-4791-9EC8-3651D794C8C6}">
-  <dimension ref="A1:T77"/>
-  <sheetFormatPr defaultRowHeight="14.5"/>
+  <dimension ref="A1:T78"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="12.54296875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="39.26953125" style="3" customWidth="1"/>
-    <col min="4" max="4" width="28.54296875" style="3" hidden="1" customWidth="1"/>
-    <col min="5" max="5" width="11.453125" customWidth="1"/>
-    <col min="6" max="6" width="18.7265625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="15.81640625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="9.81640625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="10.54296875" style="4" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="31.54296875" customWidth="1"/>
-    <col min="11" max="11" width="10.54296875" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="12.7265625" customWidth="1"/>
-    <col min="13" max="13" width="13.81640625" customWidth="1"/>
-    <col min="18" max="18" width="20.453125" hidden="1" customWidth="1"/>
-    <col min="19" max="19" width="21.54296875" hidden="1" customWidth="1"/>
+    <col min="2" max="2" width="12.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="39.28515625" style="3" customWidth="1"/>
+    <col min="4" max="4" width="28.5703125" style="3" hidden="1" customWidth="1"/>
+    <col min="5" max="5" width="11.42578125" customWidth="1"/>
+    <col min="6" max="6" width="18.7109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="15.85546875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="9.85546875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="10.5703125" style="4" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="31.5703125" customWidth="1"/>
+    <col min="11" max="11" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="12.7109375" customWidth="1"/>
+    <col min="13" max="13" width="13.85546875" customWidth="1"/>
+    <col min="18" max="18" width="20.42578125" hidden="1" customWidth="1"/>
+    <col min="19" max="19" width="21.5703125" hidden="1" customWidth="1"/>
     <col min="20" max="20" width="0" hidden="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:20" ht="26">
+    <row r="1" spans="1:20" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A1" s="27" t="s">
         <v>108</v>
       </c>
@@ -6046,7 +6055,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="2" spans="1:20" ht="37.5">
+    <row r="2" spans="1:20" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A2" s="71" t="s">
         <v>119</v>
       </c>
@@ -6096,7 +6105,7 @@
       </c>
       <c r="T2" s="16"/>
     </row>
-    <row r="3" spans="1:20" ht="29">
+    <row r="3" spans="1:20" ht="30" x14ac:dyDescent="0.25">
       <c r="A3" s="71" t="s">
         <v>126</v>
       </c>
@@ -6146,7 +6155,7 @@
       </c>
       <c r="T3" s="16"/>
     </row>
-    <row r="4" spans="1:20" ht="43.5">
+    <row r="4" spans="1:20" ht="45" x14ac:dyDescent="0.25">
       <c r="A4" s="71" t="s">
         <v>129</v>
       </c>
@@ -6196,7 +6205,7 @@
       </c>
       <c r="T4" s="16"/>
     </row>
-    <row r="5" spans="1:20" ht="43.5">
+    <row r="5" spans="1:20" ht="45" x14ac:dyDescent="0.25">
       <c r="A5" s="71" t="s">
         <v>135</v>
       </c>
@@ -6246,7 +6255,7 @@
       </c>
       <c r="T5" s="16"/>
     </row>
-    <row r="6" spans="1:20" ht="58">
+    <row r="6" spans="1:20" ht="60" x14ac:dyDescent="0.25">
       <c r="A6" s="61" t="s">
         <v>140</v>
       </c>
@@ -6296,7 +6305,7 @@
       </c>
       <c r="T6" s="16"/>
     </row>
-    <row r="7" spans="1:20" ht="43.5">
+    <row r="7" spans="1:20" ht="45" x14ac:dyDescent="0.25">
       <c r="A7" s="71" t="s">
         <v>140</v>
       </c>
@@ -6319,11 +6328,11 @@
         <v>2</v>
       </c>
       <c r="H7" s="74">
-        <f t="shared" ref="H7:H12" si="2">IF(AND(B7="Risk",ISNUMBER(F7),ISNUMBER(G7)),F7*G7,"")</f>
+        <f t="shared" ref="H7:H13" si="2">IF(AND(B7="Risk",ISNUMBER(F7),ISNUMBER(G7)),F7*G7,"")</f>
         <v>6</v>
       </c>
       <c r="I7" s="75" t="str">
-        <f t="shared" ref="I7:I12" si="3">IF(H7="","",IF(H7&gt;=15,"Red",IF(H7&gt;=8,"Amber","Green")))</f>
+        <f t="shared" ref="I7:I13" si="3">IF(H7="","",IF(H7&gt;=15,"Red",IF(H7&gt;=8,"Amber","Green")))</f>
         <v>Green</v>
       </c>
       <c r="J7" s="8" t="s">
@@ -6346,7 +6355,7 @@
       </c>
       <c r="T7" s="16"/>
     </row>
-    <row r="8" spans="1:20" ht="43.5">
+    <row r="8" spans="1:20" ht="45" x14ac:dyDescent="0.25">
       <c r="A8" s="71" t="s">
         <v>144</v>
       </c>
@@ -6396,7 +6405,7 @@
       </c>
       <c r="T8" s="16"/>
     </row>
-    <row r="9" spans="1:20" ht="43.5">
+    <row r="9" spans="1:20" ht="45" x14ac:dyDescent="0.25">
       <c r="A9" s="71" t="s">
         <v>147</v>
       </c>
@@ -6442,7 +6451,7 @@
       <c r="S9" s="16"/>
       <c r="T9" s="16"/>
     </row>
-    <row r="10" spans="1:20" ht="72.5">
+    <row r="10" spans="1:20" ht="75" x14ac:dyDescent="0.25">
       <c r="A10" s="71" t="s">
         <v>150</v>
       </c>
@@ -6492,60 +6501,62 @@
       </c>
       <c r="T10" s="16"/>
     </row>
-    <row r="11" spans="1:20" ht="29">
+    <row r="11" spans="1:20" ht="75" x14ac:dyDescent="0.25">
       <c r="A11" s="71" t="s">
-        <v>171</v>
+        <v>588</v>
       </c>
       <c r="B11" s="72" t="s">
-        <v>172</v>
+        <v>120</v>
       </c>
       <c r="C11" s="8" t="s">
-        <v>176</v>
-      </c>
-      <c r="D11" s="69" t="s">
-        <v>177</v>
-      </c>
-      <c r="E11" s="8"/>
-      <c r="F11" s="6"/>
-      <c r="G11" s="6"/>
-      <c r="H11" s="74" t="str">
+        <v>589</v>
+      </c>
+      <c r="D11" s="69"/>
+      <c r="E11" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="F11" s="73">
+        <v>4</v>
+      </c>
+      <c r="G11" s="73">
+        <v>4</v>
+      </c>
+      <c r="H11" s="74">
         <f t="shared" si="2"/>
-        <v/>
+        <v>16</v>
       </c>
       <c r="I11" s="75" t="str">
         <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="J11" s="8"/>
+        <v>Red</v>
+      </c>
+      <c r="J11" s="8" t="s">
+        <v>590</v>
+      </c>
       <c r="K11" s="37" t="s">
         <v>87</v>
       </c>
       <c r="L11" s="76">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="M11" s="76">
-        <v>46289</v>
-      </c>
-      <c r="R11" s="16" t="s">
-        <v>156</v>
-      </c>
-      <c r="S11" s="16" t="s">
-        <v>157</v>
-      </c>
+        <v>46290</v>
+      </c>
+      <c r="R11" s="16"/>
+      <c r="S11" s="16"/>
       <c r="T11" s="16"/>
     </row>
-    <row r="12" spans="1:20" ht="29">
+    <row r="12" spans="1:20" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A12" s="71" t="s">
-        <v>175</v>
+        <v>171</v>
       </c>
       <c r="B12" s="72" t="s">
         <v>172</v>
       </c>
       <c r="C12" s="8" t="s">
-        <v>179</v>
+        <v>176</v>
       </c>
       <c r="D12" s="69" t="s">
-        <v>180</v>
+        <v>177</v>
       </c>
       <c r="E12" s="8"/>
       <c r="F12" s="6"/>
@@ -6569,28 +6580,37 @@
         <v>46289</v>
       </c>
       <c r="R12" s="16" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="S12" s="16" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="T12" s="16"/>
     </row>
-    <row r="13" spans="1:20" ht="25">
+    <row r="13" spans="1:20" ht="45" x14ac:dyDescent="0.25">
       <c r="A13" s="71" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="B13" s="72" t="s">
         <v>172</v>
       </c>
       <c r="C13" s="8" t="s">
-        <v>55</v>
+        <v>179</v>
+      </c>
+      <c r="D13" s="69" t="s">
+        <v>180</v>
       </c>
       <c r="E13" s="8"/>
       <c r="F13" s="6"/>
       <c r="G13" s="6"/>
-      <c r="H13" s="6"/>
-      <c r="I13" s="77"/>
+      <c r="H13" s="74" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="I13" s="75" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
       <c r="J13" s="8"/>
       <c r="K13" s="37" t="s">
         <v>87</v>
@@ -6602,22 +6622,22 @@
         <v>46289</v>
       </c>
       <c r="R13" s="16" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="S13" s="16" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="T13" s="16"/>
     </row>
-    <row r="14" spans="1:20" ht="29">
+    <row r="14" spans="1:20" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A14" s="71" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
       <c r="B14" s="72" t="s">
         <v>172</v>
       </c>
       <c r="C14" s="8" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="E14" s="8"/>
       <c r="F14" s="6"/>
@@ -6635,29 +6655,28 @@
         <v>46289</v>
       </c>
       <c r="R14" s="16" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="S14" s="16" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="T14" s="16"/>
     </row>
-    <row r="15" spans="1:20" ht="29">
+    <row r="15" spans="1:20" ht="30" x14ac:dyDescent="0.25">
       <c r="A15" s="71" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="B15" s="72" t="s">
         <v>172</v>
       </c>
       <c r="C15" s="8" t="s">
-        <v>57</v>
-      </c>
-      <c r="D15" s="69"/>
+        <v>56</v>
+      </c>
       <c r="E15" s="8"/>
       <c r="F15" s="6"/>
       <c r="G15" s="6"/>
-      <c r="H15" s="74"/>
-      <c r="I15" s="75"/>
+      <c r="H15" s="6"/>
+      <c r="I15" s="77"/>
       <c r="J15" s="8"/>
       <c r="K15" s="37" t="s">
         <v>87</v>
@@ -6669,22 +6688,22 @@
         <v>46289</v>
       </c>
       <c r="R15" s="16" t="s">
-        <v>165</v>
+        <v>162</v>
       </c>
       <c r="S15" s="16" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
       <c r="T15" s="16"/>
     </row>
-    <row r="16" spans="1:20" ht="29">
+    <row r="16" spans="1:20" ht="30" x14ac:dyDescent="0.25">
       <c r="A16" s="71" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="B16" s="72" t="s">
         <v>172</v>
       </c>
       <c r="C16" s="8" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="D16" s="69"/>
       <c r="E16" s="8"/>
@@ -6703,22 +6722,22 @@
         <v>46289</v>
       </c>
       <c r="R16" s="16" t="s">
-        <v>169</v>
+        <v>165</v>
       </c>
       <c r="S16" s="16" t="s">
-        <v>170</v>
+        <v>166</v>
       </c>
       <c r="T16" s="16"/>
     </row>
-    <row r="17" spans="1:20" ht="58">
+    <row r="17" spans="1:20" ht="30" x14ac:dyDescent="0.25">
       <c r="A17" s="71" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="B17" s="72" t="s">
         <v>172</v>
       </c>
       <c r="C17" s="8" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="D17" s="69"/>
       <c r="E17" s="8"/>
@@ -6736,19 +6755,23 @@
       <c r="M17" s="76">
         <v>46289</v>
       </c>
-      <c r="R17" s="16"/>
-      <c r="S17" s="16"/>
+      <c r="R17" s="16" t="s">
+        <v>169</v>
+      </c>
+      <c r="S17" s="16" t="s">
+        <v>170</v>
+      </c>
       <c r="T17" s="16"/>
     </row>
-    <row r="18" spans="1:20" ht="29">
+    <row r="18" spans="1:20" ht="60" x14ac:dyDescent="0.25">
       <c r="A18" s="71" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="B18" s="72" t="s">
         <v>172</v>
       </c>
       <c r="C18" s="8" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="D18" s="69"/>
       <c r="E18" s="8"/>
@@ -6770,21 +6793,22 @@
       <c r="S18" s="16"/>
       <c r="T18" s="16"/>
     </row>
-    <row r="19" spans="1:20" ht="43.5">
+    <row r="19" spans="1:20" ht="30" x14ac:dyDescent="0.25">
       <c r="A19" s="71" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="B19" s="72" t="s">
         <v>172</v>
       </c>
       <c r="C19" s="8" t="s">
-        <v>61</v>
-      </c>
+        <v>60</v>
+      </c>
+      <c r="D19" s="69"/>
       <c r="E19" s="8"/>
       <c r="F19" s="6"/>
       <c r="G19" s="6"/>
-      <c r="H19" s="6"/>
-      <c r="I19" s="77"/>
+      <c r="H19" s="74"/>
+      <c r="I19" s="75"/>
       <c r="J19" s="8"/>
       <c r="K19" s="37" t="s">
         <v>87</v>
@@ -6799,22 +6823,21 @@
       <c r="S19" s="16"/>
       <c r="T19" s="16"/>
     </row>
-    <row r="20" spans="1:20" ht="43.5">
+    <row r="20" spans="1:20" ht="60" x14ac:dyDescent="0.25">
       <c r="A20" s="71" t="s">
-        <v>298</v>
+        <v>186</v>
       </c>
       <c r="B20" s="72" t="s">
         <v>172</v>
       </c>
       <c r="C20" s="8" t="s">
-        <v>62</v>
-      </c>
-      <c r="D20" s="69"/>
+        <v>61</v>
+      </c>
       <c r="E20" s="8"/>
       <c r="F20" s="6"/>
       <c r="G20" s="6"/>
-      <c r="H20" s="74"/>
-      <c r="I20" s="75"/>
+      <c r="H20" s="6"/>
+      <c r="I20" s="77"/>
       <c r="J20" s="8"/>
       <c r="K20" s="37" t="s">
         <v>87</v>
@@ -6829,27 +6852,23 @@
       <c r="S20" s="16"/>
       <c r="T20" s="16"/>
     </row>
-    <row r="21" spans="1:20" ht="29">
+    <row r="21" spans="1:20" ht="45" x14ac:dyDescent="0.25">
       <c r="A21" s="71" t="s">
-        <v>187</v>
+        <v>298</v>
       </c>
       <c r="B21" s="72" t="s">
-        <v>188</v>
+        <v>172</v>
       </c>
       <c r="C21" s="8" t="s">
-        <v>305</v>
-      </c>
-      <c r="D21"/>
-      <c r="E21" s="8" t="s">
-        <v>8</v>
-      </c>
+        <v>62</v>
+      </c>
+      <c r="D21" s="69"/>
+      <c r="E21" s="8"/>
       <c r="F21" s="6"/>
       <c r="G21" s="6"/>
-      <c r="H21" s="6"/>
-      <c r="I21" s="77"/>
-      <c r="J21" s="8" t="s">
-        <v>297</v>
-      </c>
+      <c r="H21" s="74"/>
+      <c r="I21" s="75"/>
+      <c r="J21" s="8"/>
       <c r="K21" s="37" t="s">
         <v>87</v>
       </c>
@@ -6863,15 +6882,15 @@
       <c r="S21" s="16"/>
       <c r="T21" s="16"/>
     </row>
-    <row r="22" spans="1:20" ht="43.5">
+    <row r="22" spans="1:20" ht="45" x14ac:dyDescent="0.25">
       <c r="A22" s="71" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="B22" s="72" t="s">
         <v>188</v>
       </c>
       <c r="C22" s="8" t="s">
-        <v>299</v>
+        <v>305</v>
       </c>
       <c r="D22"/>
       <c r="E22" s="8" t="s">
@@ -6882,7 +6901,7 @@
       <c r="H22" s="6"/>
       <c r="I22" s="77"/>
       <c r="J22" s="8" t="s">
-        <v>304</v>
+        <v>297</v>
       </c>
       <c r="K22" s="37" t="s">
         <v>87</v>
@@ -6897,26 +6916,26 @@
       <c r="S22" s="16"/>
       <c r="T22" s="16"/>
     </row>
-    <row r="23" spans="1:20" ht="43.5">
+    <row r="23" spans="1:20" ht="45" x14ac:dyDescent="0.25">
       <c r="A23" s="71" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="B23" s="72" t="s">
         <v>188</v>
       </c>
       <c r="C23" s="8" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="D23"/>
       <c r="E23" s="8" t="s">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="F23" s="6"/>
       <c r="G23" s="6"/>
       <c r="H23" s="6"/>
-      <c r="I23" s="6"/>
+      <c r="I23" s="77"/>
       <c r="J23" s="8" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="K23" s="37" t="s">
         <v>87</v>
@@ -6931,26 +6950,26 @@
       <c r="S23" s="16"/>
       <c r="T23" s="16"/>
     </row>
-    <row r="24" spans="1:20" ht="43.5">
+    <row r="24" spans="1:20" ht="45" x14ac:dyDescent="0.25">
       <c r="A24" s="71" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="B24" s="72" t="s">
         <v>188</v>
       </c>
       <c r="C24" s="8" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="D24"/>
       <c r="E24" s="8" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="F24" s="6"/>
       <c r="G24" s="6"/>
       <c r="H24" s="6"/>
       <c r="I24" s="6"/>
       <c r="J24" s="8" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="K24" s="37" t="s">
         <v>87</v>
@@ -6965,28 +6984,26 @@
       <c r="S24" s="16"/>
       <c r="T24" s="16"/>
     </row>
-    <row r="25" spans="1:20" ht="29">
+    <row r="25" spans="1:20" ht="45" x14ac:dyDescent="0.25">
       <c r="A25" s="71" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="B25" s="72" t="s">
-        <v>193</v>
+        <v>188</v>
       </c>
       <c r="C25" s="8" t="s">
-        <v>202</v>
-      </c>
-      <c r="D25" s="70" t="s">
+        <v>301</v>
+      </c>
+      <c r="D25"/>
+      <c r="E25" s="8" t="s">
         <v>6</v>
       </c>
-      <c r="E25" s="8"/>
       <c r="F25" s="6"/>
       <c r="G25" s="6"/>
-      <c r="H25" s="75" t="s">
-        <v>174</v>
-      </c>
-      <c r="I25" s="77"/>
+      <c r="H25" s="6"/>
+      <c r="I25" s="6"/>
       <c r="J25" s="8" t="s">
-        <v>194</v>
+        <v>302</v>
       </c>
       <c r="K25" s="37" t="s">
         <v>87</v>
@@ -7001,18 +7018,18 @@
       <c r="S25" s="16"/>
       <c r="T25" s="16"/>
     </row>
-    <row r="26" spans="1:20">
+    <row r="26" spans="1:20" ht="30" x14ac:dyDescent="0.25">
       <c r="A26" s="71" t="s">
-        <v>196</v>
+        <v>192</v>
       </c>
       <c r="B26" s="72" t="s">
         <v>193</v>
       </c>
       <c r="C26" s="8" t="s">
-        <v>204</v>
+        <v>202</v>
       </c>
       <c r="D26" s="70" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="E26" s="8"/>
       <c r="F26" s="6"/>
@@ -7037,24 +7054,28 @@
       <c r="S26" s="16"/>
       <c r="T26" s="16"/>
     </row>
-    <row r="27" spans="1:20" ht="58">
+    <row r="27" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A27" s="71" t="s">
-        <v>199</v>
+        <v>196</v>
       </c>
       <c r="B27" s="72" t="s">
         <v>193</v>
       </c>
       <c r="C27" s="8" t="s">
-        <v>295</v>
-      </c>
-      <c r="D27" s="60"/>
+        <v>204</v>
+      </c>
+      <c r="D27" s="70" t="s">
+        <v>9</v>
+      </c>
       <c r="E27" s="8"/>
-      <c r="F27" s="8"/>
-      <c r="G27" s="8"/>
-      <c r="H27" s="6"/>
-      <c r="I27" s="6"/>
+      <c r="F27" s="6"/>
+      <c r="G27" s="6"/>
+      <c r="H27" s="75" t="s">
+        <v>174</v>
+      </c>
+      <c r="I27" s="77"/>
       <c r="J27" s="8" t="s">
-        <v>416</v>
+        <v>194</v>
       </c>
       <c r="K27" s="37" t="s">
         <v>87</v>
@@ -7069,15 +7090,15 @@
       <c r="S27" s="16"/>
       <c r="T27" s="16"/>
     </row>
-    <row r="28" spans="1:20" ht="58">
+    <row r="28" spans="1:20" ht="60" x14ac:dyDescent="0.25">
       <c r="A28" s="71" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="B28" s="72" t="s">
         <v>193</v>
       </c>
       <c r="C28" s="8" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="D28" s="60"/>
       <c r="E28" s="8"/>
@@ -7101,36 +7122,56 @@
       <c r="S28" s="16"/>
       <c r="T28" s="16"/>
     </row>
-    <row r="29" spans="1:20">
+    <row r="29" spans="1:20" ht="60" x14ac:dyDescent="0.25">
+      <c r="A29" s="71" t="s">
+        <v>201</v>
+      </c>
+      <c r="B29" s="72" t="s">
+        <v>193</v>
+      </c>
+      <c r="C29" s="8" t="s">
+        <v>296</v>
+      </c>
+      <c r="D29" s="60"/>
+      <c r="E29" s="8"/>
+      <c r="F29" s="8"/>
+      <c r="G29" s="8"/>
+      <c r="H29" s="6"/>
+      <c r="I29" s="6"/>
+      <c r="J29" s="8" t="s">
+        <v>416</v>
+      </c>
+      <c r="K29" s="37" t="s">
+        <v>87</v>
+      </c>
+      <c r="L29" s="76">
+        <v>46289</v>
+      </c>
+      <c r="M29" s="76">
+        <v>46289</v>
+      </c>
       <c r="R29" s="16"/>
       <c r="S29" s="16"/>
       <c r="T29" s="16"/>
     </row>
-    <row r="30" spans="1:20">
+    <row r="30" spans="1:20" x14ac:dyDescent="0.25">
       <c r="R30" s="16"/>
       <c r="S30" s="16"/>
       <c r="T30" s="16"/>
     </row>
-    <row r="31" spans="1:20">
+    <row r="31" spans="1:20" x14ac:dyDescent="0.25">
       <c r="R31" s="16"/>
       <c r="S31" s="16"/>
-      <c r="T31" s="16" t="s">
-        <v>195</v>
-      </c>
-    </row>
-    <row r="32" spans="1:20">
-      <c r="C32"/>
-      <c r="D32" s="16"/>
-      <c r="F32" s="3"/>
-      <c r="G32" s="3"/>
-      <c r="I32"/>
+      <c r="T31" s="16"/>
+    </row>
+    <row r="32" spans="1:20" x14ac:dyDescent="0.25">
       <c r="R32" s="16"/>
       <c r="S32" s="16"/>
       <c r="T32" s="16" t="s">
-        <v>197</v>
-      </c>
-    </row>
-    <row r="33" spans="1:20">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="33" spans="1:20" x14ac:dyDescent="0.25">
       <c r="C33"/>
       <c r="D33" s="16"/>
       <c r="F33" s="3"/>
@@ -7139,10 +7180,10 @@
       <c r="R33" s="16"/>
       <c r="S33" s="16"/>
       <c r="T33" s="16" t="s">
-        <v>198</v>
-      </c>
-    </row>
-    <row r="34" spans="1:20">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="34" spans="1:20" x14ac:dyDescent="0.25">
       <c r="C34"/>
       <c r="D34" s="16"/>
       <c r="F34" s="3"/>
@@ -7151,253 +7192,265 @@
       <c r="R34" s="16"/>
       <c r="S34" s="16"/>
       <c r="T34" s="16" t="s">
-        <v>200</v>
-      </c>
-    </row>
-    <row r="35" spans="1:20" ht="25">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="35" spans="1:20" x14ac:dyDescent="0.25">
       <c r="C35"/>
+      <c r="D35" s="16"/>
       <c r="F35" s="3"/>
       <c r="G35" s="3"/>
       <c r="I35"/>
       <c r="R35" s="16"/>
       <c r="S35" s="16"/>
       <c r="T35" s="16" t="s">
-        <v>203</v>
-      </c>
-    </row>
-    <row r="36" spans="1:20">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="36" spans="1:20" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="C36"/>
       <c r="F36" s="3"/>
       <c r="G36" s="3"/>
+      <c r="I36"/>
       <c r="R36" s="16"/>
       <c r="S36" s="16"/>
       <c r="T36" s="16" t="s">
-        <v>205</v>
-      </c>
-    </row>
-    <row r="37" spans="1:20">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="37" spans="1:20" x14ac:dyDescent="0.25">
       <c r="F37" s="3"/>
       <c r="G37" s="3"/>
       <c r="R37" s="16"/>
       <c r="S37" s="16"/>
       <c r="T37" s="16" t="s">
-        <v>206</v>
-      </c>
-    </row>
-    <row r="38" spans="1:20">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="38" spans="1:20" x14ac:dyDescent="0.25">
       <c r="F38" s="3"/>
       <c r="G38" s="3"/>
-    </row>
-    <row r="39" spans="1:20">
-      <c r="A39" s="14"/>
-      <c r="B39" s="13"/>
-      <c r="D39" s="59"/>
-      <c r="E39" s="13"/>
+      <c r="R38" s="16"/>
+      <c r="S38" s="16"/>
+      <c r="T38" s="16" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="39" spans="1:20" x14ac:dyDescent="0.25">
       <c r="F39" s="3"/>
       <c r="G39" s="3"/>
-      <c r="H39" s="13"/>
-      <c r="I39" s="49"/>
-      <c r="K39" s="13"/>
-      <c r="L39" s="13"/>
-      <c r="M39" s="13"/>
-      <c r="R39" s="13"/>
-      <c r="S39" s="13"/>
-      <c r="T39" s="13"/>
-    </row>
-    <row r="40" spans="1:20">
+    </row>
+    <row r="40" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A40" s="14"/>
+      <c r="B40" s="13"/>
+      <c r="D40" s="59"/>
+      <c r="E40" s="13"/>
       <c r="F40" s="3"/>
       <c r="G40" s="3"/>
-    </row>
-    <row r="41" spans="1:20">
+      <c r="H40" s="13"/>
+      <c r="I40" s="49"/>
+      <c r="K40" s="13"/>
+      <c r="L40" s="13"/>
+      <c r="M40" s="13"/>
+      <c r="R40" s="13"/>
+      <c r="S40" s="13"/>
+      <c r="T40" s="13"/>
+    </row>
+    <row r="41" spans="1:20" x14ac:dyDescent="0.25">
       <c r="F41" s="3"/>
       <c r="G41" s="3"/>
     </row>
-    <row r="42" spans="1:20">
+    <row r="42" spans="1:20" x14ac:dyDescent="0.25">
       <c r="F42" s="3"/>
       <c r="G42" s="3"/>
     </row>
-    <row r="43" spans="1:20">
+    <row r="43" spans="1:20" x14ac:dyDescent="0.25">
       <c r="F43" s="3"/>
       <c r="G43" s="3"/>
     </row>
-    <row r="44" spans="1:20">
+    <row r="44" spans="1:20" x14ac:dyDescent="0.25">
       <c r="F44" s="3"/>
       <c r="G44" s="3"/>
     </row>
-    <row r="45" spans="1:20">
+    <row r="45" spans="1:20" x14ac:dyDescent="0.25">
       <c r="F45" s="3"/>
       <c r="G45" s="3"/>
     </row>
-    <row r="46" spans="1:20">
+    <row r="46" spans="1:20" x14ac:dyDescent="0.25">
       <c r="F46" s="3"/>
       <c r="G46" s="3"/>
     </row>
-    <row r="47" spans="1:20">
+    <row r="47" spans="1:20" x14ac:dyDescent="0.25">
       <c r="F47" s="3"/>
       <c r="G47" s="3"/>
     </row>
-    <row r="48" spans="1:20">
+    <row r="48" spans="1:20" x14ac:dyDescent="0.25">
       <c r="F48" s="3"/>
       <c r="G48" s="3"/>
     </row>
-    <row r="49" spans="2:7">
+    <row r="49" spans="2:7" x14ac:dyDescent="0.25">
       <c r="F49" s="3"/>
       <c r="G49" s="3"/>
     </row>
-    <row r="50" spans="2:7">
-      <c r="B50" t="s">
-        <v>120</v>
-      </c>
-      <c r="C50" s="3" t="s">
-        <v>294</v>
-      </c>
+    <row r="50" spans="2:7" x14ac:dyDescent="0.25">
       <c r="F50" s="3"/>
       <c r="G50" s="3"/>
     </row>
-    <row r="51" spans="2:7">
+    <row r="51" spans="2:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="B51" t="s">
+        <v>120</v>
+      </c>
+      <c r="C51" s="3" t="s">
+        <v>294</v>
+      </c>
       <c r="F51" s="3"/>
       <c r="G51" s="3"/>
     </row>
-    <row r="52" spans="2:7">
+    <row r="52" spans="2:7" x14ac:dyDescent="0.25">
       <c r="F52" s="3"/>
       <c r="G52" s="3"/>
     </row>
-    <row r="53" spans="2:7">
+    <row r="53" spans="2:7" x14ac:dyDescent="0.25">
       <c r="F53" s="3"/>
       <c r="G53" s="3"/>
     </row>
-    <row r="54" spans="2:7">
+    <row r="54" spans="2:7" x14ac:dyDescent="0.25">
       <c r="F54" s="3"/>
       <c r="G54" s="3"/>
     </row>
-    <row r="55" spans="2:7">
+    <row r="55" spans="2:7" x14ac:dyDescent="0.25">
       <c r="F55" s="3"/>
       <c r="G55" s="3"/>
     </row>
-    <row r="56" spans="2:7">
+    <row r="56" spans="2:7" x14ac:dyDescent="0.25">
       <c r="F56" s="3"/>
       <c r="G56" s="3"/>
     </row>
-    <row r="57" spans="2:7">
+    <row r="57" spans="2:7" x14ac:dyDescent="0.25">
       <c r="F57" s="3"/>
       <c r="G57" s="3"/>
     </row>
-    <row r="58" spans="2:7">
+    <row r="58" spans="2:7" x14ac:dyDescent="0.25">
       <c r="F58" s="3"/>
       <c r="G58" s="3"/>
     </row>
-    <row r="59" spans="2:7">
+    <row r="59" spans="2:7" x14ac:dyDescent="0.25">
       <c r="F59" s="3"/>
       <c r="G59" s="3"/>
     </row>
-    <row r="60" spans="2:7">
+    <row r="60" spans="2:7" x14ac:dyDescent="0.25">
       <c r="F60" s="3"/>
       <c r="G60" s="3"/>
     </row>
-    <row r="61" spans="2:7">
+    <row r="61" spans="2:7" x14ac:dyDescent="0.25">
       <c r="F61" s="3"/>
       <c r="G61" s="3"/>
     </row>
-    <row r="62" spans="2:7">
+    <row r="62" spans="2:7" x14ac:dyDescent="0.25">
       <c r="F62" s="3"/>
       <c r="G62" s="3"/>
     </row>
-    <row r="63" spans="2:7">
+    <row r="63" spans="2:7" x14ac:dyDescent="0.25">
       <c r="F63" s="3"/>
       <c r="G63" s="3"/>
     </row>
-    <row r="64" spans="2:7">
+    <row r="64" spans="2:7" x14ac:dyDescent="0.25">
       <c r="F64" s="3"/>
       <c r="G64" s="3"/>
     </row>
-    <row r="65" spans="4:7">
+    <row r="65" spans="4:7" x14ac:dyDescent="0.25">
       <c r="F65" s="3"/>
       <c r="G65" s="3"/>
     </row>
-    <row r="66" spans="4:7">
+    <row r="66" spans="4:7" x14ac:dyDescent="0.25">
       <c r="F66" s="3"/>
       <c r="G66" s="3"/>
     </row>
-    <row r="67" spans="4:7">
+    <row r="67" spans="4:7" x14ac:dyDescent="0.25">
       <c r="F67" s="3"/>
       <c r="G67" s="3"/>
     </row>
-    <row r="68" spans="4:7">
+    <row r="68" spans="4:7" x14ac:dyDescent="0.25">
       <c r="F68" s="3"/>
       <c r="G68" s="3"/>
     </row>
-    <row r="69" spans="4:7">
+    <row r="69" spans="4:7" x14ac:dyDescent="0.25">
       <c r="F69" s="3"/>
       <c r="G69" s="3"/>
     </row>
-    <row r="70" spans="4:7">
+    <row r="70" spans="4:7" x14ac:dyDescent="0.25">
       <c r="F70" s="3"/>
       <c r="G70" s="3"/>
     </row>
-    <row r="71" spans="4:7">
+    <row r="71" spans="4:7" x14ac:dyDescent="0.25">
       <c r="F71" s="3"/>
       <c r="G71" s="3"/>
     </row>
-    <row r="72" spans="4:7">
+    <row r="72" spans="4:7" x14ac:dyDescent="0.25">
       <c r="F72" s="3"/>
       <c r="G72" s="3"/>
     </row>
-    <row r="73" spans="4:7">
-      <c r="D73" s="3" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="74" spans="4:7">
+    <row r="73" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="F73" s="3"/>
+      <c r="G73" s="3"/>
+    </row>
+    <row r="74" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D74" s="3" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="75" spans="4:7">
+    <row r="75" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D75" s="3" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="76" spans="4:7">
+    <row r="76" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D76" s="3" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="77" spans="4:7">
+    <row r="77" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D77" s="3" t="s">
         <v>8</v>
       </c>
     </row>
+    <row r="78" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="D78" s="3" t="s">
+        <v>8</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M37" xr:uid="{B61A661B-79AD-4791-9EC8-3651D794C8C6}"/>
-  <conditionalFormatting sqref="H25:H26">
-    <cfRule type="cellIs" dxfId="16" priority="34" operator="equal">
+  <autoFilter ref="A1:M38" xr:uid="{B61A661B-79AD-4791-9EC8-3651D794C8C6}"/>
+  <conditionalFormatting sqref="H26:H27">
+    <cfRule type="cellIs" dxfId="12" priority="34" operator="equal">
       <formula>"Red"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="15" priority="35" operator="equal">
+    <cfRule type="cellIs" dxfId="11" priority="35" operator="equal">
       <formula>"Amber"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="14" priority="36" operator="equal">
+    <cfRule type="cellIs" dxfId="10" priority="36" operator="equal">
       <formula>"Green"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I2:I12">
-    <cfRule type="cellIs" dxfId="13" priority="10" operator="equal">
+  <conditionalFormatting sqref="I2:I13">
+    <cfRule type="cellIs" dxfId="9" priority="10" operator="equal">
       <formula>"Red"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="12" priority="11" operator="equal">
+    <cfRule type="cellIs" dxfId="8" priority="11" operator="equal">
       <formula>"Amber"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="11" priority="12" operator="equal">
+    <cfRule type="cellIs" dxfId="7" priority="12" operator="equal">
       <formula>"Green"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I15:I18 I20">
-    <cfRule type="cellIs" dxfId="10" priority="70" operator="equal">
+  <conditionalFormatting sqref="I16:I19 I21">
+    <cfRule type="cellIs" dxfId="6" priority="70" operator="equal">
       <formula>"Red"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="9" priority="71" operator="equal">
+    <cfRule type="cellIs" dxfId="5" priority="71" operator="equal">
       <formula>"Amber"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="8" priority="72" operator="equal">
+    <cfRule type="cellIs" dxfId="4" priority="72" operator="equal">
       <formula>"Green"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -7446,7 +7499,7 @@
               </fill>
             </x14:dxf>
           </x14:cfRule>
-          <xm:sqref>B2:B28</xm:sqref>
+          <xm:sqref>B2:B29</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
           <x14:cfRule type="cellIs" priority="6" operator="equal" id="{344CC581-A1A3-486A-9628-9C3640970D2A}">
@@ -7489,7 +7542,7 @@
               </fill>
             </x14:dxf>
           </x14:cfRule>
-          <xm:sqref>K2:K28</xm:sqref>
+          <xm:sqref>K2:K29</xm:sqref>
         </x14:conditionalFormatting>
       </x14:conditionalFormattings>
     </ext>
@@ -7499,13 +7552,13 @@
           <x14:formula1>
             <xm:f>'Team votes &amp; Misc Info'!$J$2:$J$5</xm:f>
           </x14:formula1>
-          <xm:sqref>K2:K28</xm:sqref>
+          <xm:sqref>K2:K29</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{70105738-C97C-43BB-80BE-8021B63D21DF}">
           <x14:formula1>
             <xm:f>'Team votes &amp; Misc Info'!$L$2:$L$5</xm:f>
           </x14:formula1>
-          <xm:sqref>B2:B28</xm:sqref>
+          <xm:sqref>B2:B29</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -7516,17 +7569,17 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FA348513-37C3-4823-B24D-B6F996329F0C}">
   <dimension ref="A1:F17"/>
-  <sheetFormatPr defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="16.453125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="16.42578125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="23" customWidth="1"/>
-    <col min="3" max="3" width="12.81640625" customWidth="1"/>
-    <col min="4" max="4" width="14.81640625" customWidth="1"/>
-    <col min="5" max="5" width="10.26953125" customWidth="1"/>
-    <col min="6" max="6" width="10.453125" customWidth="1"/>
+    <col min="3" max="3" width="12.85546875" customWidth="1"/>
+    <col min="4" max="4" width="14.85546875" customWidth="1"/>
+    <col min="5" max="5" width="10.28515625" customWidth="1"/>
+    <col min="6" max="6" width="10.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="27" t="s">
         <v>255</v>
       </c>
@@ -7538,7 +7591,7 @@
       <c r="E1" s="27"/>
       <c r="F1" s="27"/>
     </row>
-    <row r="2" spans="1:6">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="27"/>
       <c r="B2" s="27" t="s">
         <v>207</v>
@@ -7556,7 +7609,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="3" spans="1:6">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="23" t="s">
         <v>212</v>
       </c>
@@ -7581,7 +7634,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:6">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" s="23" t="s">
         <v>213</v>
       </c>
@@ -7606,7 +7659,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:6">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="23" t="s">
         <v>214</v>
       </c>
@@ -7631,7 +7684,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:6">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="23" t="s">
         <v>215</v>
       </c>
@@ -7656,7 +7709,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:6">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" s="23" t="s">
         <v>216</v>
       </c>
@@ -7681,22 +7734,22 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:6" ht="32.5" customHeight="1">
-      <c r="A9" s="126" t="s">
+    <row r="9" spans="1:6" ht="32.450000000000003" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="120" t="s">
         <v>217</v>
       </c>
-      <c r="B9" s="126"/>
-      <c r="C9" s="126"/>
-      <c r="D9" s="126"/>
-      <c r="E9" s="126"/>
-      <c r="F9" s="126"/>
-    </row>
-    <row r="11" spans="1:6" ht="15.5">
+      <c r="B9" s="120"/>
+      <c r="C9" s="120"/>
+      <c r="D9" s="120"/>
+      <c r="E9" s="120"/>
+      <c r="F9" s="120"/>
+    </row>
+    <row r="11" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A11" s="21" t="s">
         <v>218</v>
       </c>
     </row>
-    <row r="12" spans="1:6">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" s="27" t="s">
         <v>112</v>
       </c>
@@ -7704,7 +7757,7 @@
         <v>219</v>
       </c>
     </row>
-    <row r="13" spans="1:6">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" s="42">
         <v>1</v>
       </c>
@@ -7712,7 +7765,7 @@
         <v>220</v>
       </c>
     </row>
-    <row r="14" spans="1:6">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" s="42">
         <v>2</v>
       </c>
@@ -7720,7 +7773,7 @@
         <v>221</v>
       </c>
     </row>
-    <row r="15" spans="1:6">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" s="42">
         <v>3</v>
       </c>
@@ -7728,7 +7781,7 @@
         <v>222</v>
       </c>
     </row>
-    <row r="16" spans="1:6">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" s="42">
         <v>4</v>
       </c>
@@ -7736,7 +7789,7 @@
         <v>223</v>
       </c>
     </row>
-    <row r="17" spans="1:2" ht="29">
+    <row r="17" spans="1:2" ht="30" x14ac:dyDescent="0.25">
       <c r="A17" s="42">
         <v>5</v>
       </c>
@@ -7755,20 +7808,20 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{569F1412-D6F6-4C33-BE23-573808AF6A8E}">
   <dimension ref="A1:X61"/>
-  <sheetFormatPr defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="9.54296875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="52.453125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.54296875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="6.26953125" customWidth="1"/>
-    <col min="5" max="5" width="61.1796875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="15.54296875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="7.81640625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="8.81640625" bestFit="1" customWidth="1"/>
-    <col min="9" max="10" width="9.1796875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="52.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.5703125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="6.28515625" customWidth="1"/>
+    <col min="5" max="5" width="61.140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="15.5703125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="7.85546875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="8.85546875" bestFit="1" customWidth="1"/>
+    <col min="9" max="10" width="9.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="30" customHeight="1">
+    <row r="1" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="82" t="s">
         <v>331</v>
       </c>
@@ -7800,7 +7853,7 @@
         <v>337</v>
       </c>
     </row>
-    <row r="2" spans="1:10">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" s="81" t="s">
         <v>338</v>
       </c>
@@ -7832,7 +7885,7 @@
         <v>46290</v>
       </c>
     </row>
-    <row r="3" spans="1:10">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3" s="81" t="s">
         <v>338</v>
       </c>
@@ -7864,7 +7917,7 @@
         <v>46290</v>
       </c>
     </row>
-    <row r="4" spans="1:10">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A4" s="81" t="s">
         <v>338</v>
       </c>
@@ -7896,7 +7949,7 @@
         <v>46290</v>
       </c>
     </row>
-    <row r="5" spans="1:10">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A5" s="81" t="s">
         <v>338</v>
       </c>
@@ -7928,7 +7981,7 @@
         <v>46290</v>
       </c>
     </row>
-    <row r="6" spans="1:10">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A6" s="81" t="s">
         <v>338</v>
       </c>
@@ -7960,7 +8013,7 @@
         <v>46290</v>
       </c>
     </row>
-    <row r="7" spans="1:10">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A7" s="81" t="s">
         <v>338</v>
       </c>
@@ -7992,7 +8045,7 @@
         <v>46290</v>
       </c>
     </row>
-    <row r="8" spans="1:10">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A8" s="81" t="s">
         <v>338</v>
       </c>
@@ -8024,7 +8077,7 @@
         <v>46290</v>
       </c>
     </row>
-    <row r="9" spans="1:10">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A9" s="81" t="s">
         <v>338</v>
       </c>
@@ -8056,7 +8109,7 @@
         <v>46290</v>
       </c>
     </row>
-    <row r="10" spans="1:10">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A10" s="81" t="s">
         <v>362</v>
       </c>
@@ -8088,7 +8141,7 @@
         <v>46290</v>
       </c>
     </row>
-    <row r="11" spans="1:10">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A11" s="81" t="s">
         <v>362</v>
       </c>
@@ -8120,7 +8173,7 @@
         <v>46290</v>
       </c>
     </row>
-    <row r="12" spans="1:10">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A12" s="81" t="s">
         <v>362</v>
       </c>
@@ -8152,7 +8205,7 @@
         <v>46290</v>
       </c>
     </row>
-    <row r="13" spans="1:10">
+    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A13" s="81" t="s">
         <v>362</v>
       </c>
@@ -8184,7 +8237,7 @@
         <v>46290</v>
       </c>
     </row>
-    <row r="14" spans="1:10">
+    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A14" s="81" t="s">
         <v>362</v>
       </c>
@@ -8216,7 +8269,7 @@
         <v>46290</v>
       </c>
     </row>
-    <row r="15" spans="1:10">
+    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A15" s="81" t="s">
         <v>362</v>
       </c>
@@ -8248,7 +8301,7 @@
         <v>46290</v>
       </c>
     </row>
-    <row r="16" spans="1:10">
+    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A16" s="81" t="s">
         <v>362</v>
       </c>
@@ -8280,7 +8333,7 @@
         <v>46290</v>
       </c>
     </row>
-    <row r="17" spans="1:10">
+    <row r="17" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A17" s="81" t="s">
         <v>362</v>
       </c>
@@ -8312,7 +8365,7 @@
         <v>46290</v>
       </c>
     </row>
-    <row r="18" spans="1:10">
+    <row r="18" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A18" s="81" t="s">
         <v>362</v>
       </c>
@@ -8344,7 +8397,7 @@
         <v>46290</v>
       </c>
     </row>
-    <row r="19" spans="1:10">
+    <row r="19" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A19" s="81" t="s">
         <v>362</v>
       </c>
@@ -8376,7 +8429,7 @@
         <v>46290</v>
       </c>
     </row>
-    <row r="20" spans="1:10">
+    <row r="20" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A20" s="81" t="s">
         <v>362</v>
       </c>
@@ -8408,7 +8461,7 @@
         <v>46290</v>
       </c>
     </row>
-    <row r="21" spans="1:10">
+    <row r="21" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A21" s="81" t="s">
         <v>362</v>
       </c>
@@ -8440,7 +8493,7 @@
         <v>46290</v>
       </c>
     </row>
-    <row r="22" spans="1:10">
+    <row r="22" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A22" s="81" t="s">
         <v>362</v>
       </c>
@@ -8472,7 +8525,7 @@
         <v>46290</v>
       </c>
     </row>
-    <row r="23" spans="1:10">
+    <row r="23" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A23" s="81" t="s">
         <v>362</v>
       </c>
@@ -8504,7 +8557,7 @@
         <v>46290</v>
       </c>
     </row>
-    <row r="24" spans="1:10">
+    <row r="24" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A24" s="81" t="s">
         <v>362</v>
       </c>
@@ -8536,7 +8589,7 @@
         <v>46290</v>
       </c>
     </row>
-    <row r="25" spans="1:10">
+    <row r="25" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A25" s="81" t="s">
         <v>362</v>
       </c>
@@ -8568,7 +8621,7 @@
         <v>46290</v>
       </c>
     </row>
-    <row r="26" spans="1:10">
+    <row r="26" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A26" s="81" t="s">
         <v>362</v>
       </c>
@@ -8600,7 +8653,7 @@
         <v>46290</v>
       </c>
     </row>
-    <row r="27" spans="1:10">
+    <row r="27" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A27" s="81" t="s">
         <v>362</v>
       </c>
@@ -8632,7 +8685,7 @@
         <v>46290</v>
       </c>
     </row>
-    <row r="28" spans="1:10">
+    <row r="28" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A28" s="81" t="s">
         <v>362</v>
       </c>
@@ -8664,7 +8717,7 @@
         <v>46290</v>
       </c>
     </row>
-    <row r="29" spans="1:10">
+    <row r="29" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A29" s="81" t="s">
         <v>403</v>
       </c>
@@ -8696,7 +8749,7 @@
         <v>46290</v>
       </c>
     </row>
-    <row r="30" spans="1:10">
+    <row r="30" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A30" s="81" t="s">
         <v>403</v>
       </c>
@@ -8728,7 +8781,7 @@
         <v>46290</v>
       </c>
     </row>
-    <row r="31" spans="1:10">
+    <row r="31" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A31" s="81" t="s">
         <v>403</v>
       </c>
@@ -8760,7 +8813,7 @@
         <v>46290</v>
       </c>
     </row>
-    <row r="32" spans="1:10">
+    <row r="32" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A32" s="81" t="s">
         <v>403</v>
       </c>
@@ -8792,7 +8845,7 @@
         <v>46290</v>
       </c>
     </row>
-    <row r="33" spans="1:24">
+    <row r="33" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A33" s="81" t="s">
         <v>403</v>
       </c>
@@ -8824,7 +8877,7 @@
         <v>46290</v>
       </c>
     </row>
-    <row r="34" spans="1:24">
+    <row r="34" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A34" s="81" t="s">
         <v>403</v>
       </c>
@@ -8856,7 +8909,7 @@
         <v>46290</v>
       </c>
     </row>
-    <row r="35" spans="1:24">
+    <row r="35" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A35" s="81" t="s">
         <v>403</v>
       </c>
@@ -8888,97 +8941,97 @@
         <v>46290</v>
       </c>
     </row>
-    <row r="42" spans="1:24" ht="14.5" customHeight="1">
-      <c r="A42" s="120" t="s">
+    <row r="42" spans="1:24" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A42" s="121" t="s">
         <v>418</v>
       </c>
-      <c r="B42" s="120"/>
-      <c r="C42" s="120"/>
-      <c r="D42" s="120"/>
-      <c r="E42" s="120"/>
-      <c r="F42" s="120"/>
-      <c r="G42" s="120"/>
-      <c r="I42" s="121" t="s">
+      <c r="B42" s="121"/>
+      <c r="C42" s="121"/>
+      <c r="D42" s="121"/>
+      <c r="E42" s="121"/>
+      <c r="F42" s="121"/>
+      <c r="G42" s="121"/>
+      <c r="I42" s="122" t="s">
         <v>419</v>
       </c>
-      <c r="J42" s="122"/>
-      <c r="K42" s="122"/>
-      <c r="L42" s="122"/>
-      <c r="M42" s="122"/>
-      <c r="N42" s="122"/>
-      <c r="O42" s="122"/>
-      <c r="P42" s="122"/>
-      <c r="Q42" s="122"/>
-      <c r="R42" s="122"/>
-      <c r="S42" s="122"/>
-      <c r="T42" s="122"/>
-      <c r="U42" s="122"/>
-      <c r="V42" s="122"/>
-      <c r="W42" s="122"/>
-      <c r="X42" s="122"/>
-    </row>
-    <row r="43" spans="1:24">
-      <c r="A43" s="120"/>
-      <c r="B43" s="120"/>
-      <c r="C43" s="120"/>
-      <c r="D43" s="120"/>
-      <c r="E43" s="120"/>
-      <c r="F43" s="120"/>
-      <c r="G43" s="120"/>
-      <c r="I43" s="121"/>
-      <c r="J43" s="122"/>
-      <c r="K43" s="122"/>
-      <c r="L43" s="122"/>
-      <c r="M43" s="122"/>
-      <c r="N43" s="122"/>
-      <c r="O43" s="122"/>
-      <c r="P43" s="122"/>
-      <c r="Q43" s="122"/>
-      <c r="R43" s="122"/>
-      <c r="S43" s="122"/>
-      <c r="T43" s="122"/>
-      <c r="U43" s="122"/>
-      <c r="V43" s="122"/>
-      <c r="W43" s="122"/>
-      <c r="X43" s="122"/>
-    </row>
-    <row r="60" spans="9:24" ht="14.5" customHeight="1">
-      <c r="I60" s="120" t="s">
+      <c r="J42" s="123"/>
+      <c r="K42" s="123"/>
+      <c r="L42" s="123"/>
+      <c r="M42" s="123"/>
+      <c r="N42" s="123"/>
+      <c r="O42" s="123"/>
+      <c r="P42" s="123"/>
+      <c r="Q42" s="123"/>
+      <c r="R42" s="123"/>
+      <c r="S42" s="123"/>
+      <c r="T42" s="123"/>
+      <c r="U42" s="123"/>
+      <c r="V42" s="123"/>
+      <c r="W42" s="123"/>
+      <c r="X42" s="123"/>
+    </row>
+    <row r="43" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="A43" s="121"/>
+      <c r="B43" s="121"/>
+      <c r="C43" s="121"/>
+      <c r="D43" s="121"/>
+      <c r="E43" s="121"/>
+      <c r="F43" s="121"/>
+      <c r="G43" s="121"/>
+      <c r="I43" s="122"/>
+      <c r="J43" s="123"/>
+      <c r="K43" s="123"/>
+      <c r="L43" s="123"/>
+      <c r="M43" s="123"/>
+      <c r="N43" s="123"/>
+      <c r="O43" s="123"/>
+      <c r="P43" s="123"/>
+      <c r="Q43" s="123"/>
+      <c r="R43" s="123"/>
+      <c r="S43" s="123"/>
+      <c r="T43" s="123"/>
+      <c r="U43" s="123"/>
+      <c r="V43" s="123"/>
+      <c r="W43" s="123"/>
+      <c r="X43" s="123"/>
+    </row>
+    <row r="60" spans="9:24" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="I60" s="121" t="s">
         <v>420</v>
       </c>
-      <c r="J60" s="120"/>
-      <c r="K60" s="120"/>
-      <c r="L60" s="120"/>
-      <c r="M60" s="120"/>
-      <c r="N60" s="120"/>
-      <c r="O60" s="120"/>
-      <c r="P60" s="120"/>
-      <c r="Q60" s="120"/>
-      <c r="R60" s="120"/>
-      <c r="S60" s="120"/>
-      <c r="T60" s="120"/>
-      <c r="U60" s="120"/>
-      <c r="V60" s="120"/>
-      <c r="W60" s="120"/>
-      <c r="X60" s="120"/>
-    </row>
-    <row r="61" spans="9:24">
-      <c r="I61" s="120"/>
-      <c r="J61" s="120"/>
-      <c r="K61" s="120"/>
-      <c r="L61" s="120"/>
-      <c r="M61" s="120"/>
-      <c r="N61" s="120"/>
-      <c r="O61" s="120"/>
-      <c r="P61" s="120"/>
-      <c r="Q61" s="120"/>
-      <c r="R61" s="120"/>
-      <c r="S61" s="120"/>
-      <c r="T61" s="120"/>
-      <c r="U61" s="120"/>
-      <c r="V61" s="120"/>
-      <c r="W61" s="120"/>
-      <c r="X61" s="120"/>
+      <c r="J60" s="121"/>
+      <c r="K60" s="121"/>
+      <c r="L60" s="121"/>
+      <c r="M60" s="121"/>
+      <c r="N60" s="121"/>
+      <c r="O60" s="121"/>
+      <c r="P60" s="121"/>
+      <c r="Q60" s="121"/>
+      <c r="R60" s="121"/>
+      <c r="S60" s="121"/>
+      <c r="T60" s="121"/>
+      <c r="U60" s="121"/>
+      <c r="V60" s="121"/>
+      <c r="W60" s="121"/>
+      <c r="X60" s="121"/>
+    </row>
+    <row r="61" spans="9:24" x14ac:dyDescent="0.25">
+      <c r="I61" s="121"/>
+      <c r="J61" s="121"/>
+      <c r="K61" s="121"/>
+      <c r="L61" s="121"/>
+      <c r="M61" s="121"/>
+      <c r="N61" s="121"/>
+      <c r="O61" s="121"/>
+      <c r="P61" s="121"/>
+      <c r="Q61" s="121"/>
+      <c r="R61" s="121"/>
+      <c r="S61" s="121"/>
+      <c r="T61" s="121"/>
+      <c r="U61" s="121"/>
+      <c r="V61" s="121"/>
+      <c r="W61" s="121"/>
+      <c r="X61" s="121"/>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -8995,49 +9048,49 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DE7F1919-2543-40B0-86E7-ADC6C70417C2}">
   <dimension ref="A1:H145"/>
-  <sheetFormatPr defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="17.7265625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="7.1796875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="8.81640625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="33.81640625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="69.7265625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="122.81640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="17.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="7.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="8.85546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="33.85546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="69.7109375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="122.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="14.5" customHeight="1">
-      <c r="A1" s="125" t="s">
+    <row r="1" spans="1:8" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="126" t="s">
         <v>54</v>
       </c>
-      <c r="B1" s="125"/>
-      <c r="C1" s="125"/>
-      <c r="D1" s="125"/>
-      <c r="E1" s="125"/>
+      <c r="B1" s="126"/>
+      <c r="C1" s="126"/>
+      <c r="D1" s="126"/>
+      <c r="E1" s="126"/>
       <c r="H1" s="1"/>
     </row>
-    <row r="3" spans="1:8">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="B3" s="123" t="s">
+      <c r="B3" s="124" t="s">
         <v>429</v>
       </c>
-      <c r="C3" s="124"/>
-      <c r="D3" s="124"/>
-      <c r="E3" s="124"/>
-    </row>
-    <row r="4" spans="1:8">
+      <c r="C3" s="125"/>
+      <c r="D3" s="125"/>
+      <c r="E3" s="125"/>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="B4" s="123" t="s">
+      <c r="B4" s="124" t="s">
         <v>430</v>
       </c>
-      <c r="C4" s="124"/>
-      <c r="D4" s="124"/>
-      <c r="E4" s="124"/>
-    </row>
-    <row r="5" spans="1:8">
+      <c r="C4" s="125"/>
+      <c r="D4" s="125"/>
+      <c r="E4" s="125"/>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>41</v>
       </c>
@@ -9054,7 +9107,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="6" spans="1:8">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>431</v>
       </c>
@@ -9071,7 +9124,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="7" spans="1:8">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>434</v>
       </c>
@@ -9088,7 +9141,7 @@
         <v>436</v>
       </c>
     </row>
-    <row r="8" spans="1:8">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>437</v>
       </c>
@@ -9102,7 +9155,7 @@
         <v>438</v>
       </c>
     </row>
-    <row r="9" spans="1:8">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>439</v>
       </c>
@@ -9116,7 +9169,7 @@
         <v>441</v>
       </c>
     </row>
-    <row r="10" spans="1:8">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>442</v>
       </c>
@@ -9130,7 +9183,7 @@
         <v>444</v>
       </c>
     </row>
-    <row r="11" spans="1:8">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>445</v>
       </c>
@@ -9141,7 +9194,7 @@
         <v>446</v>
       </c>
     </row>
-    <row r="12" spans="1:8">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>447</v>
       </c>
@@ -9158,7 +9211,7 @@
         <v>450</v>
       </c>
     </row>
-    <row r="13" spans="1:8">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>451</v>
       </c>
@@ -9169,7 +9222,7 @@
         <v>452</v>
       </c>
     </row>
-    <row r="14" spans="1:8">
+    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>453</v>
       </c>
@@ -9180,7 +9233,7 @@
         <v>454</v>
       </c>
     </row>
-    <row r="15" spans="1:8">
+    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>455</v>
       </c>
@@ -9197,7 +9250,7 @@
         <v>457</v>
       </c>
     </row>
-    <row r="16" spans="1:8">
+    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>458</v>
       </c>
@@ -9211,7 +9264,7 @@
         <v>460</v>
       </c>
     </row>
-    <row r="17" spans="1:5">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>461</v>
       </c>
@@ -9225,7 +9278,7 @@
         <v>462</v>
       </c>
     </row>
-    <row r="18" spans="1:5">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>463</v>
       </c>
@@ -9239,7 +9292,7 @@
         <v>465</v>
       </c>
     </row>
-    <row r="19" spans="1:5">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>466</v>
       </c>
@@ -9253,7 +9306,7 @@
         <v>467</v>
       </c>
     </row>
-    <row r="20" spans="1:5">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>468</v>
       </c>
@@ -9264,7 +9317,7 @@
         <v>469</v>
       </c>
     </row>
-    <row r="21" spans="1:5">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>470</v>
       </c>
@@ -9275,29 +9328,29 @@
         <v>472</v>
       </c>
     </row>
-    <row r="23" spans="1:5">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="B23" s="123" t="s">
+      <c r="B23" s="124" t="s">
         <v>473</v>
       </c>
-      <c r="C23" s="124"/>
-      <c r="D23" s="124"/>
-      <c r="E23" s="124"/>
-    </row>
-    <row r="24" spans="1:5">
+      <c r="C23" s="125"/>
+      <c r="D23" s="125"/>
+      <c r="E23" s="125"/>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="B24" s="123" t="s">
+      <c r="B24" s="124" t="s">
         <v>474</v>
       </c>
-      <c r="C24" s="124"/>
-      <c r="D24" s="124"/>
-      <c r="E24" s="124"/>
-    </row>
-    <row r="25" spans="1:5">
+      <c r="C24" s="125"/>
+      <c r="D24" s="125"/>
+      <c r="E24" s="125"/>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" s="1" t="s">
         <v>41</v>
       </c>
@@ -9314,7 +9367,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="26" spans="1:5">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>434</v>
       </c>
@@ -9331,7 +9384,7 @@
         <v>475</v>
       </c>
     </row>
-    <row r="27" spans="1:5">
+    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>476</v>
       </c>
@@ -9342,7 +9395,7 @@
         <v>477</v>
       </c>
     </row>
-    <row r="28" spans="1:5">
+    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>478</v>
       </c>
@@ -9353,7 +9406,7 @@
         <v>479</v>
       </c>
     </row>
-    <row r="29" spans="1:5">
+    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>480</v>
       </c>
@@ -9364,7 +9417,7 @@
         <v>481</v>
       </c>
     </row>
-    <row r="30" spans="1:5">
+    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>482</v>
       </c>
@@ -9375,29 +9428,29 @@
         <v>483</v>
       </c>
     </row>
-    <row r="32" spans="1:5">
+    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A32" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="B32" s="123" t="s">
+      <c r="B32" s="124" t="s">
         <v>484</v>
       </c>
-      <c r="C32" s="124"/>
-      <c r="D32" s="124"/>
-      <c r="E32" s="124"/>
-    </row>
-    <row r="33" spans="1:5">
+      <c r="C32" s="125"/>
+      <c r="D32" s="125"/>
+      <c r="E32" s="125"/>
+    </row>
+    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A33" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="B33" s="123" t="s">
+      <c r="B33" s="124" t="s">
         <v>485</v>
       </c>
-      <c r="C33" s="124"/>
-      <c r="D33" s="124"/>
-      <c r="E33" s="124"/>
-    </row>
-    <row r="34" spans="1:5">
+      <c r="C33" s="125"/>
+      <c r="D33" s="125"/>
+      <c r="E33" s="125"/>
+    </row>
+    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A34" s="1" t="s">
         <v>41</v>
       </c>
@@ -9414,7 +9467,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="35" spans="1:5">
+    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>439</v>
       </c>
@@ -9431,7 +9484,7 @@
         <v>486</v>
       </c>
     </row>
-    <row r="36" spans="1:5">
+    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>49</v>
       </c>
@@ -9445,29 +9498,29 @@
         <v>50</v>
       </c>
     </row>
-    <row r="38" spans="1:5">
+    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A38" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="B38" s="123" t="s">
+      <c r="B38" s="124" t="s">
         <v>487</v>
       </c>
-      <c r="C38" s="124"/>
-      <c r="D38" s="124"/>
-      <c r="E38" s="124"/>
-    </row>
-    <row r="39" spans="1:5">
+      <c r="C38" s="125"/>
+      <c r="D38" s="125"/>
+      <c r="E38" s="125"/>
+    </row>
+    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A39" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="B39" s="123" t="s">
+      <c r="B39" s="124" t="s">
         <v>488</v>
       </c>
-      <c r="C39" s="124"/>
-      <c r="D39" s="124"/>
-      <c r="E39" s="124"/>
-    </row>
-    <row r="40" spans="1:5">
+      <c r="C39" s="125"/>
+      <c r="D39" s="125"/>
+      <c r="E39" s="125"/>
+    </row>
+    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A40" s="1" t="s">
         <v>41</v>
       </c>
@@ -9484,7 +9537,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="41" spans="1:5">
+    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>442</v>
       </c>
@@ -9501,7 +9554,7 @@
         <v>489</v>
       </c>
     </row>
-    <row r="42" spans="1:5">
+    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>490</v>
       </c>
@@ -9515,29 +9568,29 @@
         <v>491</v>
       </c>
     </row>
-    <row r="44" spans="1:5">
+    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A44" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="B44" s="123" t="s">
+      <c r="B44" s="124" t="s">
         <v>492</v>
       </c>
-      <c r="C44" s="124"/>
-      <c r="D44" s="124"/>
-      <c r="E44" s="124"/>
-    </row>
-    <row r="45" spans="1:5">
+      <c r="C44" s="125"/>
+      <c r="D44" s="125"/>
+      <c r="E44" s="125"/>
+    </row>
+    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A45" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="B45" s="123" t="s">
+      <c r="B45" s="124" t="s">
         <v>493</v>
       </c>
-      <c r="C45" s="124"/>
-      <c r="D45" s="124"/>
-      <c r="E45" s="124"/>
-    </row>
-    <row r="46" spans="1:5">
+      <c r="C45" s="125"/>
+      <c r="D45" s="125"/>
+      <c r="E45" s="125"/>
+    </row>
+    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A46" s="1" t="s">
         <v>41</v>
       </c>
@@ -9554,7 +9607,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="47" spans="1:5">
+    <row r="47" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>494</v>
       </c>
@@ -9571,7 +9624,7 @@
         <v>495</v>
       </c>
     </row>
-    <row r="48" spans="1:5">
+    <row r="48" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>52</v>
       </c>
@@ -9588,29 +9641,29 @@
         <v>497</v>
       </c>
     </row>
-    <row r="50" spans="1:5">
+    <row r="50" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A50" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="B50" s="123" t="s">
+      <c r="B50" s="124" t="s">
         <v>498</v>
       </c>
-      <c r="C50" s="124"/>
-      <c r="D50" s="124"/>
-      <c r="E50" s="124"/>
-    </row>
-    <row r="51" spans="1:5">
+      <c r="C50" s="125"/>
+      <c r="D50" s="125"/>
+      <c r="E50" s="125"/>
+    </row>
+    <row r="51" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A51" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="B51" s="123" t="s">
+      <c r="B51" s="124" t="s">
         <v>499</v>
       </c>
-      <c r="C51" s="124"/>
-      <c r="D51" s="124"/>
-      <c r="E51" s="124"/>
-    </row>
-    <row r="52" spans="1:5">
+      <c r="C51" s="125"/>
+      <c r="D51" s="125"/>
+      <c r="E51" s="125"/>
+    </row>
+    <row r="52" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A52" s="1" t="s">
         <v>41</v>
       </c>
@@ -9627,7 +9680,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="53" spans="1:5">
+    <row r="53" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
         <v>500</v>
       </c>
@@ -9644,7 +9697,7 @@
         <v>501</v>
       </c>
     </row>
-    <row r="54" spans="1:5">
+    <row r="54" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
         <v>431</v>
       </c>
@@ -9658,7 +9711,7 @@
         <v>502</v>
       </c>
     </row>
-    <row r="55" spans="1:5">
+    <row r="55" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
         <v>494</v>
       </c>
@@ -9672,7 +9725,7 @@
         <v>503</v>
       </c>
     </row>
-    <row r="56" spans="1:5">
+    <row r="56" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
         <v>504</v>
       </c>
@@ -9683,29 +9736,29 @@
         <v>505</v>
       </c>
     </row>
-    <row r="58" spans="1:5">
+    <row r="58" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A58" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="B58" s="123" t="s">
+      <c r="B58" s="124" t="s">
         <v>506</v>
       </c>
-      <c r="C58" s="124"/>
-      <c r="D58" s="124"/>
-      <c r="E58" s="124"/>
-    </row>
-    <row r="59" spans="1:5">
+      <c r="C58" s="125"/>
+      <c r="D58" s="125"/>
+      <c r="E58" s="125"/>
+    </row>
+    <row r="59" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A59" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="B59" s="123" t="s">
+      <c r="B59" s="124" t="s">
         <v>507</v>
       </c>
-      <c r="C59" s="124"/>
-      <c r="D59" s="124"/>
-      <c r="E59" s="124"/>
-    </row>
-    <row r="60" spans="1:5">
+      <c r="C59" s="125"/>
+      <c r="D59" s="125"/>
+      <c r="E59" s="125"/>
+    </row>
+    <row r="60" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A60" s="1" t="s">
         <v>41</v>
       </c>
@@ -9722,7 +9775,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="61" spans="1:5">
+    <row r="61" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
         <v>508</v>
       </c>
@@ -9739,7 +9792,7 @@
         <v>509</v>
       </c>
     </row>
-    <row r="62" spans="1:5">
+    <row r="62" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
         <v>510</v>
       </c>
@@ -9753,29 +9806,29 @@
         <v>511</v>
       </c>
     </row>
-    <row r="64" spans="1:5">
+    <row r="64" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A64" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="B64" s="123" t="s">
+      <c r="B64" s="124" t="s">
         <v>512</v>
       </c>
-      <c r="C64" s="124"/>
-      <c r="D64" s="124"/>
-      <c r="E64" s="124"/>
-    </row>
-    <row r="65" spans="1:5">
+      <c r="C64" s="125"/>
+      <c r="D64" s="125"/>
+      <c r="E64" s="125"/>
+    </row>
+    <row r="65" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A65" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="B65" s="123" t="s">
+      <c r="B65" s="124" t="s">
         <v>513</v>
       </c>
-      <c r="C65" s="124"/>
-      <c r="D65" s="124"/>
-      <c r="E65" s="124"/>
-    </row>
-    <row r="66" spans="1:5">
+      <c r="C65" s="125"/>
+      <c r="D65" s="125"/>
+      <c r="E65" s="125"/>
+    </row>
+    <row r="66" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A66" s="1" t="s">
         <v>41</v>
       </c>
@@ -9792,7 +9845,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="67" spans="1:5">
+    <row r="67" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
         <v>514</v>
       </c>
@@ -9809,7 +9862,7 @@
         <v>515</v>
       </c>
     </row>
-    <row r="68" spans="1:5">
+    <row r="68" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
         <v>431</v>
       </c>
@@ -9823,7 +9876,7 @@
         <v>502</v>
       </c>
     </row>
-    <row r="69" spans="1:5">
+    <row r="69" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
         <v>508</v>
       </c>
@@ -9837,7 +9890,7 @@
         <v>516</v>
       </c>
     </row>
-    <row r="70" spans="1:5">
+    <row r="70" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
         <v>517</v>
       </c>
@@ -9848,29 +9901,29 @@
         <v>518</v>
       </c>
     </row>
-    <row r="72" spans="1:5">
+    <row r="72" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A72" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="B72" s="123" t="s">
+      <c r="B72" s="124" t="s">
         <v>519</v>
       </c>
-      <c r="C72" s="124"/>
-      <c r="D72" s="124"/>
-      <c r="E72" s="124"/>
-    </row>
-    <row r="73" spans="1:5">
+      <c r="C72" s="125"/>
+      <c r="D72" s="125"/>
+      <c r="E72" s="125"/>
+    </row>
+    <row r="73" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A73" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="B73" s="123" t="s">
+      <c r="B73" s="124" t="s">
         <v>520</v>
       </c>
-      <c r="C73" s="124"/>
-      <c r="D73" s="124"/>
-      <c r="E73" s="124"/>
-    </row>
-    <row r="74" spans="1:5">
+      <c r="C73" s="125"/>
+      <c r="D73" s="125"/>
+      <c r="E73" s="125"/>
+    </row>
+    <row r="74" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A74" s="1" t="s">
         <v>41</v>
       </c>
@@ -9887,7 +9940,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="75" spans="1:5">
+    <row r="75" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
         <v>521</v>
       </c>
@@ -9904,7 +9957,7 @@
         <v>522</v>
       </c>
     </row>
-    <row r="76" spans="1:5">
+    <row r="76" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
         <v>523</v>
       </c>
@@ -9918,29 +9971,29 @@
         <v>524</v>
       </c>
     </row>
-    <row r="78" spans="1:5">
+    <row r="78" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A78" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="B78" s="123" t="s">
+      <c r="B78" s="124" t="s">
         <v>525</v>
       </c>
-      <c r="C78" s="124"/>
-      <c r="D78" s="124"/>
-      <c r="E78" s="124"/>
-    </row>
-    <row r="79" spans="1:5">
+      <c r="C78" s="125"/>
+      <c r="D78" s="125"/>
+      <c r="E78" s="125"/>
+    </row>
+    <row r="79" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A79" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="B79" s="123" t="s">
+      <c r="B79" s="124" t="s">
         <v>526</v>
       </c>
-      <c r="C79" s="124"/>
-      <c r="D79" s="124"/>
-      <c r="E79" s="124"/>
-    </row>
-    <row r="80" spans="1:5">
+      <c r="C79" s="125"/>
+      <c r="D79" s="125"/>
+      <c r="E79" s="125"/>
+    </row>
+    <row r="80" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A80" s="1" t="s">
         <v>41</v>
       </c>
@@ -9957,7 +10010,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="81" spans="1:5">
+    <row r="81" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
         <v>527</v>
       </c>
@@ -9974,7 +10027,7 @@
         <v>528</v>
       </c>
     </row>
-    <row r="82" spans="1:5">
+    <row r="82" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
         <v>431</v>
       </c>
@@ -9988,7 +10041,7 @@
         <v>502</v>
       </c>
     </row>
-    <row r="83" spans="1:5">
+    <row r="83" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
         <v>521</v>
       </c>
@@ -10002,7 +10055,7 @@
         <v>529</v>
       </c>
     </row>
-    <row r="84" spans="1:5">
+    <row r="84" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
         <v>530</v>
       </c>
@@ -10013,7 +10066,7 @@
         <v>531</v>
       </c>
     </row>
-    <row r="85" spans="1:5">
+    <row r="85" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
         <v>532</v>
       </c>
@@ -10024,7 +10077,7 @@
         <v>533</v>
       </c>
     </row>
-    <row r="86" spans="1:5">
+    <row r="86" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
         <v>534</v>
       </c>
@@ -10035,7 +10088,7 @@
         <v>535</v>
       </c>
     </row>
-    <row r="87" spans="1:5">
+    <row r="87" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
         <v>536</v>
       </c>
@@ -10046,29 +10099,29 @@
         <v>537</v>
       </c>
     </row>
-    <row r="89" spans="1:5">
+    <row r="89" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A89" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="B89" s="123" t="s">
+      <c r="B89" s="124" t="s">
         <v>538</v>
       </c>
-      <c r="C89" s="124"/>
-      <c r="D89" s="124"/>
-      <c r="E89" s="124"/>
-    </row>
-    <row r="90" spans="1:5">
+      <c r="C89" s="125"/>
+      <c r="D89" s="125"/>
+      <c r="E89" s="125"/>
+    </row>
+    <row r="90" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A90" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="B90" s="123" t="s">
+      <c r="B90" s="124" t="s">
         <v>539</v>
       </c>
-      <c r="C90" s="124"/>
-      <c r="D90" s="124"/>
-      <c r="E90" s="124"/>
-    </row>
-    <row r="91" spans="1:5">
+      <c r="C90" s="125"/>
+      <c r="D90" s="125"/>
+      <c r="E90" s="125"/>
+    </row>
+    <row r="91" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A91" s="1" t="s">
         <v>41</v>
       </c>
@@ -10085,7 +10138,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="92" spans="1:5">
+    <row r="92" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
         <v>540</v>
       </c>
@@ -10102,7 +10155,7 @@
         <v>541</v>
       </c>
     </row>
-    <row r="93" spans="1:5">
+    <row r="93" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
         <v>53</v>
       </c>
@@ -10116,7 +10169,7 @@
         <v>542</v>
       </c>
     </row>
-    <row r="94" spans="1:5">
+    <row r="94" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
         <v>543</v>
       </c>
@@ -10130,7 +10183,7 @@
         <v>545</v>
       </c>
     </row>
-    <row r="95" spans="1:5">
+    <row r="95" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A95" t="s">
         <v>546</v>
       </c>
@@ -10144,29 +10197,29 @@
         <v>547</v>
       </c>
     </row>
-    <row r="97" spans="1:5">
+    <row r="97" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A97" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="B97" s="123" t="s">
+      <c r="B97" s="124" t="s">
         <v>548</v>
       </c>
-      <c r="C97" s="124"/>
-      <c r="D97" s="124"/>
-      <c r="E97" s="124"/>
-    </row>
-    <row r="98" spans="1:5">
+      <c r="C97" s="125"/>
+      <c r="D97" s="125"/>
+      <c r="E97" s="125"/>
+    </row>
+    <row r="98" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A98" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="B98" s="123" t="s">
+      <c r="B98" s="124" t="s">
         <v>549</v>
       </c>
-      <c r="C98" s="124"/>
-      <c r="D98" s="124"/>
-      <c r="E98" s="124"/>
-    </row>
-    <row r="99" spans="1:5">
+      <c r="C98" s="125"/>
+      <c r="D98" s="125"/>
+      <c r="E98" s="125"/>
+    </row>
+    <row r="99" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A99" s="1" t="s">
         <v>41</v>
       </c>
@@ -10183,7 +10236,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="100" spans="1:5">
+    <row r="100" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
         <v>550</v>
       </c>
@@ -10200,7 +10253,7 @@
         <v>528</v>
       </c>
     </row>
-    <row r="101" spans="1:5">
+    <row r="101" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A101" t="s">
         <v>431</v>
       </c>
@@ -10217,7 +10270,7 @@
         <v>551</v>
       </c>
     </row>
-    <row r="102" spans="1:5">
+    <row r="102" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A102" t="s">
         <v>540</v>
       </c>
@@ -10234,7 +10287,7 @@
         <v>553</v>
       </c>
     </row>
-    <row r="103" spans="1:5">
+    <row r="103" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A103" t="s">
         <v>532</v>
       </c>
@@ -10245,7 +10298,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="104" spans="1:5">
+    <row r="104" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A104" t="s">
         <v>534</v>
       </c>
@@ -10256,7 +10309,7 @@
         <v>535</v>
       </c>
     </row>
-    <row r="105" spans="1:5">
+    <row r="105" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A105" t="s">
         <v>536</v>
       </c>
@@ -10267,29 +10320,29 @@
         <v>537</v>
       </c>
     </row>
-    <row r="107" spans="1:5">
+    <row r="107" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A107" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="B107" s="123" t="s">
+      <c r="B107" s="124" t="s">
         <v>555</v>
       </c>
-      <c r="C107" s="124"/>
-      <c r="D107" s="124"/>
-      <c r="E107" s="124"/>
-    </row>
-    <row r="108" spans="1:5">
+      <c r="C107" s="125"/>
+      <c r="D107" s="125"/>
+      <c r="E107" s="125"/>
+    </row>
+    <row r="108" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A108" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="B108" s="123" t="s">
+      <c r="B108" s="124" t="s">
         <v>556</v>
       </c>
-      <c r="C108" s="124"/>
-      <c r="D108" s="124"/>
-      <c r="E108" s="124"/>
-    </row>
-    <row r="109" spans="1:5">
+      <c r="C108" s="125"/>
+      <c r="D108" s="125"/>
+      <c r="E108" s="125"/>
+    </row>
+    <row r="109" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A109" s="1" t="s">
         <v>41</v>
       </c>
@@ -10306,7 +10359,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="110" spans="1:5">
+    <row r="110" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A110" t="s">
         <v>557</v>
       </c>
@@ -10323,7 +10376,7 @@
         <v>558</v>
       </c>
     </row>
-    <row r="111" spans="1:5">
+    <row r="111" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A111" t="s">
         <v>431</v>
       </c>
@@ -10337,7 +10390,7 @@
         <v>502</v>
       </c>
     </row>
-    <row r="112" spans="1:5">
+    <row r="112" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A112" t="s">
         <v>559</v>
       </c>
@@ -10348,7 +10401,7 @@
         <v>560</v>
       </c>
     </row>
-    <row r="113" spans="1:5">
+    <row r="113" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A113" t="s">
         <v>561</v>
       </c>
@@ -10359,29 +10412,29 @@
         <v>562</v>
       </c>
     </row>
-    <row r="115" spans="1:5">
+    <row r="115" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A115" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="B115" s="123" t="s">
+      <c r="B115" s="124" t="s">
         <v>563</v>
       </c>
-      <c r="C115" s="124"/>
-      <c r="D115" s="124"/>
-      <c r="E115" s="124"/>
-    </row>
-    <row r="116" spans="1:5">
+      <c r="C115" s="125"/>
+      <c r="D115" s="125"/>
+      <c r="E115" s="125"/>
+    </row>
+    <row r="116" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A116" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="B116" s="123" t="s">
+      <c r="B116" s="124" t="s">
         <v>564</v>
       </c>
-      <c r="C116" s="124"/>
-      <c r="D116" s="124"/>
-      <c r="E116" s="124"/>
-    </row>
-    <row r="117" spans="1:5">
+      <c r="C116" s="125"/>
+      <c r="D116" s="125"/>
+      <c r="E116" s="125"/>
+    </row>
+    <row r="117" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A117" s="1" t="s">
         <v>41</v>
       </c>
@@ -10398,7 +10451,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="118" spans="1:5">
+    <row r="118" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A118" t="s">
         <v>565</v>
       </c>
@@ -10415,7 +10468,7 @@
         <v>566</v>
       </c>
     </row>
-    <row r="119" spans="1:5">
+    <row r="119" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A119" t="s">
         <v>431</v>
       </c>
@@ -10429,7 +10482,7 @@
         <v>502</v>
       </c>
     </row>
-    <row r="120" spans="1:5">
+    <row r="120" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A120" t="s">
         <v>567</v>
       </c>
@@ -10443,7 +10496,7 @@
         <v>569</v>
       </c>
     </row>
-    <row r="121" spans="1:5">
+    <row r="121" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A121" t="s">
         <v>559</v>
       </c>
@@ -10454,7 +10507,7 @@
         <v>570</v>
       </c>
     </row>
-    <row r="122" spans="1:5">
+    <row r="122" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A122" t="s">
         <v>561</v>
       </c>
@@ -10465,29 +10518,29 @@
         <v>571</v>
       </c>
     </row>
-    <row r="124" spans="1:5">
+    <row r="124" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A124" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="B124" s="123" t="s">
+      <c r="B124" s="124" t="s">
         <v>572</v>
       </c>
-      <c r="C124" s="124"/>
-      <c r="D124" s="124"/>
-      <c r="E124" s="124"/>
-    </row>
-    <row r="125" spans="1:5">
+      <c r="C124" s="125"/>
+      <c r="D124" s="125"/>
+      <c r="E124" s="125"/>
+    </row>
+    <row r="125" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A125" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="B125" s="123" t="s">
+      <c r="B125" s="124" t="s">
         <v>573</v>
       </c>
-      <c r="C125" s="124"/>
-      <c r="D125" s="124"/>
-      <c r="E125" s="124"/>
-    </row>
-    <row r="126" spans="1:5">
+      <c r="C125" s="125"/>
+      <c r="D125" s="125"/>
+      <c r="E125" s="125"/>
+    </row>
+    <row r="126" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A126" s="1" t="s">
         <v>41</v>
       </c>
@@ -10504,7 +10557,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="127" spans="1:5">
+    <row r="127" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A127" t="s">
         <v>574</v>
       </c>
@@ -10521,7 +10574,7 @@
         <v>575</v>
       </c>
     </row>
-    <row r="128" spans="1:5">
+    <row r="128" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A128" t="s">
         <v>431</v>
       </c>
@@ -10535,7 +10588,7 @@
         <v>502</v>
       </c>
     </row>
-    <row r="129" spans="1:5">
+    <row r="129" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A129" t="s">
         <v>576</v>
       </c>
@@ -10546,7 +10599,7 @@
         <v>577</v>
       </c>
     </row>
-    <row r="130" spans="1:5">
+    <row r="130" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A130" t="s">
         <v>534</v>
       </c>
@@ -10557,7 +10610,7 @@
         <v>578</v>
       </c>
     </row>
-    <row r="131" spans="1:5">
+    <row r="131" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A131" t="s">
         <v>536</v>
       </c>
@@ -10568,29 +10621,29 @@
         <v>579</v>
       </c>
     </row>
-    <row r="133" spans="1:5">
+    <row r="133" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A133" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="B133" s="123" t="s">
+      <c r="B133" s="124" t="s">
         <v>580</v>
       </c>
-      <c r="C133" s="124"/>
-      <c r="D133" s="124"/>
-      <c r="E133" s="124"/>
-    </row>
-    <row r="134" spans="1:5">
+      <c r="C133" s="125"/>
+      <c r="D133" s="125"/>
+      <c r="E133" s="125"/>
+    </row>
+    <row r="134" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A134" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="B134" s="123" t="s">
+      <c r="B134" s="124" t="s">
         <v>581</v>
       </c>
-      <c r="C134" s="124"/>
-      <c r="D134" s="124"/>
-      <c r="E134" s="124"/>
-    </row>
-    <row r="135" spans="1:5">
+      <c r="C134" s="125"/>
+      <c r="D134" s="125"/>
+      <c r="E134" s="125"/>
+    </row>
+    <row r="135" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A135" s="1" t="s">
         <v>41</v>
       </c>
@@ -10607,7 +10660,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="136" spans="1:5">
+    <row r="136" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A136" t="s">
         <v>437</v>
       </c>
@@ -10624,7 +10677,7 @@
         <v>582</v>
       </c>
     </row>
-    <row r="137" spans="1:5">
+    <row r="137" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A137" t="s">
         <v>434</v>
       </c>
@@ -10641,7 +10694,7 @@
         <v>583</v>
       </c>
     </row>
-    <row r="138" spans="1:5">
+    <row r="138" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A138" t="s">
         <v>468</v>
       </c>
@@ -10652,7 +10705,7 @@
         <v>469</v>
       </c>
     </row>
-    <row r="139" spans="1:5">
+    <row r="139" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A139" t="s">
         <v>455</v>
       </c>
@@ -10666,7 +10719,7 @@
         <v>457</v>
       </c>
     </row>
-    <row r="140" spans="1:5">
+    <row r="140" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A140" t="s">
         <v>458</v>
       </c>
@@ -10680,7 +10733,7 @@
         <v>460</v>
       </c>
     </row>
-    <row r="141" spans="1:5">
+    <row r="141" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A141" t="s">
         <v>461</v>
       </c>
@@ -10691,7 +10744,7 @@
         <v>584</v>
       </c>
     </row>
-    <row r="142" spans="1:5">
+    <row r="142" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A142" t="s">
         <v>463</v>
       </c>
@@ -10702,7 +10755,7 @@
         <v>465</v>
       </c>
     </row>
-    <row r="143" spans="1:5">
+    <row r="143" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A143" t="s">
         <v>466</v>
       </c>
@@ -10713,7 +10766,7 @@
         <v>467</v>
       </c>
     </row>
-    <row r="144" spans="1:5">
+    <row r="144" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A144" t="s">
         <v>470</v>
       </c>
@@ -10724,7 +10777,7 @@
         <v>472</v>
       </c>
     </row>
-    <row r="145" spans="1:5">
+    <row r="145" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A145" t="s">
         <v>585</v>
       </c>
@@ -10740,19 +10793,7 @@
     </row>
   </sheetData>
   <mergeCells count="33">
-    <mergeCell ref="B125:E125"/>
-    <mergeCell ref="B133:E133"/>
-    <mergeCell ref="B134:E134"/>
-    <mergeCell ref="B107:E107"/>
-    <mergeCell ref="B108:E108"/>
-    <mergeCell ref="B115:E115"/>
-    <mergeCell ref="B116:E116"/>
-    <mergeCell ref="B124:E124"/>
-    <mergeCell ref="B39:E39"/>
-    <mergeCell ref="B45:E45"/>
-    <mergeCell ref="B44:E44"/>
-    <mergeCell ref="B97:E97"/>
-    <mergeCell ref="B98:E98"/>
+    <mergeCell ref="B89:E89"/>
     <mergeCell ref="A1:E1"/>
     <mergeCell ref="B38:E38"/>
     <mergeCell ref="B24:E24"/>
@@ -10761,6 +10802,11 @@
     <mergeCell ref="B3:E3"/>
     <mergeCell ref="B4:E4"/>
     <mergeCell ref="B33:E33"/>
+    <mergeCell ref="B39:E39"/>
+    <mergeCell ref="B45:E45"/>
+    <mergeCell ref="B44:E44"/>
+    <mergeCell ref="B97:E97"/>
+    <mergeCell ref="B98:E98"/>
     <mergeCell ref="B50:E50"/>
     <mergeCell ref="B51:E51"/>
     <mergeCell ref="B78:E78"/>
@@ -10772,7 +10818,14 @@
     <mergeCell ref="B58:E58"/>
     <mergeCell ref="B64:E64"/>
     <mergeCell ref="B65:E65"/>
-    <mergeCell ref="B89:E89"/>
+    <mergeCell ref="B125:E125"/>
+    <mergeCell ref="B133:E133"/>
+    <mergeCell ref="B134:E134"/>
+    <mergeCell ref="B107:E107"/>
+    <mergeCell ref="B108:E108"/>
+    <mergeCell ref="B115:E115"/>
+    <mergeCell ref="B116:E116"/>
+    <mergeCell ref="B124:E124"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -10782,14 +10835,14 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{42F8DE2A-76E6-452A-AE90-13C80C3D40F2}">
   <dimension ref="A1:E32"/>
-  <sheetFormatPr defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="57.26953125" customWidth="1"/>
-    <col min="2" max="2" width="18.7265625" customWidth="1"/>
-    <col min="3" max="3" width="19.7265625" customWidth="1"/>
+    <col min="1" max="1" width="57.28515625" customWidth="1"/>
+    <col min="2" max="2" width="18.7109375" customWidth="1"/>
+    <col min="3" max="3" width="19.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>20</v>
       </c>
@@ -10800,7 +10853,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="2" spans="1:5">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>24</v>
       </c>
@@ -10811,7 +10864,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:5">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>26</v>
       </c>
@@ -10819,7 +10872,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="4" spans="1:5" ht="29">
+    <row r="4" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A4" s="5" t="s">
         <v>25</v>
       </c>
@@ -10830,7 +10883,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="5" spans="1:5">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>27</v>
       </c>
@@ -10841,57 +10894,57 @@
         <v>8</v>
       </c>
     </row>
-    <row r="6" spans="1:5">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="8" spans="1:5">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="9" spans="1:5">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="13" spans="1:5">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="17" spans="1:1" ht="101.5">
+    <row r="17" spans="1:1" ht="105" x14ac:dyDescent="0.25">
       <c r="A17" s="3" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="22" spans="1:1">
+    <row r="22" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="23" spans="1:1">
+    <row r="23" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="24" spans="1:1">
+    <row r="24" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="26" spans="1:1">
+    <row r="26" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="29" spans="1:1">
+    <row r="29" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="32" spans="1:1">
+    <row r="32" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>94</v>
       </c>

</xml_diff>